<commit_message>
Ui modifications in huddle detailPanel and Onboarding Page Laxmi 7/10/2026
</commit_message>
<xml_diff>
--- a/Action_Items_Tracking_Sheet_Formatted.xlsx
+++ b/Action_Items_Tracking_Sheet_Formatted.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AITO-Recovered\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D739102-6192-45D1-A6A3-24AB4C7A0EA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE14822-E10F-4877-B962-0E74C7B86137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="199">
   <si>
     <t>Action Items &amp; Work Hours Tracking Log</t>
   </si>
@@ -1540,34 +1540,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Need to work on data part (I found same topic appears  in multiple week places in the in-app </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>role path page
-**Task: Correct the Role Path role → week → topic data mapping using the updated Excel as the source of
- truth, trace and fix the underlying duplication/mismatch, and validate all roles without modifying 
-any unrelated UI, functionality, or files.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
     <t>only in in app
 modify the 
 data.</t>
@@ -1617,6 +1589,181 @@
     <t>in-app
 prompt
 in teams chat</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Need to work on data part (I found same topic appears  in multiple week places in the in-app </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>role path page
+Task: Correct the Role Path role → week → topic data mapping using the updated Excel as the source of
+ truth, trace and fix the underlying duplication/mismatch, and validate all roles without modifying 
+any unrelated UI, functionality, or files.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Investigate alternatives to the current `access_as_user` scope approach, as obtaining the
+ required client/admin consent is expected to take around 3 months.
+Explore and evaluate alternative authentication approaches that can allow the 
+application to go live sooner while maintaining the required application functionality.</t>
+  </si>
+  <si>
+    <t>6hrs</t>
+  </si>
+  <si>
+    <t>Investigate the current access_as_user authentication, APIM, Private App Service, and Microsoft
+ Graph/OBO flow, and identify the limitations with the current approach.
+Explore alternative architectures such as SWA → APIM → Private App Service and 
+determine the best feasible approach that can address the current authentication/consent 
+issue without breaking existing functionality.</t>
+  </si>
+  <si>
+    <t>3. Rename the Step 01 card from "Onboarding" to "Onboarding / Orientation" so users understand
+ what this step is for.</t>
+  </si>
+  <si>
+    <t>done in both
+in-app &amp;
+main app.</t>
+  </si>
+  <si>
+    <r>
+      <t>Remove the</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> “Effort” </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">section from the three cards under </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">“One motion. Three connected steps” </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>and professionally reorganize the remaining card content without affecting other pages or components.  In 
+HuddleOnboardingExperience.tsx file.</t>
+    </r>
+  </si>
+  <si>
+    <t>verify in main
+ app</t>
+  </si>
+  <si>
+    <t>verify in main
+app</t>
+  </si>
+  <si>
+    <t>Update the "Huddle Details panel" by placing the "HTML" button at the top and "Generate Huddle" below it, while preserving their respective styling and existing functionality.</t>
+  </si>
+  <si>
+    <t>Gone through video to understand the requirements</t>
+  </si>
+  <si>
+    <t>Swap the “What brings you here today?” and “Top 5 Agents” sections, reorganize the Top 5 Agents into a spacious 2-column layout, and fit all agents within the existing card space without increasing the overall section height.</t>
+  </si>
+  <si>
+    <t>need to 
+implment in main app</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Remove </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>Step 6 – “Join your first huddle”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> from the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>“Before you begin”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> section of the 
+onboarding page without affecting other features.
+b.Simplify the "Readiness Checklist" by replacing “Complete AI Fundamentals” with “Top 5 MCAPS Agents Training” and combining it with "Recommended Resources" to reduce the checklist to approximately four items.</t>
+    </r>
+  </si>
+  <si>
+    <t>Renamed and repositioned "Generate Huddle" as a "Facilitator-specific experience", with a subtle CTA and appropriate access flow for different user roles.</t>
+  </si>
+  <si>
+    <t>verfiy in main app</t>
   </si>
 </sst>
 </file>
@@ -1880,7 +2027,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1939,9 +2086,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1979,8 +2123,44 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="14" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2000,59 +2180,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="15" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2321,7 +2465,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H157"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2334,14 +2478,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:6" ht="21.75" customHeight="1">
       <c r="A2" s="3" t="s">
@@ -2367,13 +2511,13 @@
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="49">
+      <c r="B3" s="44">
         <v>46260</v>
       </c>
-      <c r="C3" s="51" t="s">
+      <c r="C3" s="46" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="55">
+      <c r="D3" s="43">
         <v>6.5</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -2387,9 +2531,9 @@
       <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="49"/>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
+      <c r="B4" s="44"/>
+      <c r="C4" s="44"/>
+      <c r="D4" s="44"/>
       <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
@@ -2401,9 +2545,9 @@
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
+      <c r="B5" s="44"/>
+      <c r="C5" s="44"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
@@ -2415,9 +2559,9 @@
       <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="49"/>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
       <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
@@ -2429,9 +2573,9 @@
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
       <c r="E7" s="4" t="s">
         <v>13</v>
       </c>
@@ -2443,10 +2587,10 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="46">
+      <c r="B8" s="45">
         <v>46261</v>
       </c>
-      <c r="C8" s="45" t="s">
+      <c r="C8" s="47" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -2463,8 +2607,8 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="46"/>
-      <c r="C9" s="46"/>
+      <c r="B9" s="45"/>
+      <c r="C9" s="45"/>
       <c r="D9" s="1" t="s">
         <v>111</v>
       </c>
@@ -2479,8 +2623,8 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="46"/>
-      <c r="C10" s="46"/>
+      <c r="B10" s="45"/>
+      <c r="C10" s="45"/>
       <c r="D10" s="1" t="s">
         <v>99</v>
       </c>
@@ -2495,8 +2639,8 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
+      <c r="B11" s="45"/>
+      <c r="C11" s="45"/>
       <c r="D11" s="1" t="s">
         <v>101</v>
       </c>
@@ -2511,8 +2655,8 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="46"/>
-      <c r="C12" s="46"/>
+      <c r="B12" s="45"/>
+      <c r="C12" s="45"/>
       <c r="D12" s="1" t="s">
         <v>109</v>
       </c>
@@ -2527,8 +2671,8 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="46"/>
-      <c r="C13" s="46"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
       <c r="D13" s="1" t="s">
         <v>109</v>
       </c>
@@ -2543,8 +2687,8 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="C14" s="46"/>
+      <c r="B14" s="45"/>
+      <c r="C14" s="45"/>
       <c r="D14" s="1" t="s">
         <v>99</v>
       </c>
@@ -2559,8 +2703,8 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="46"/>
+      <c r="B15" s="45"/>
+      <c r="C15" s="45"/>
       <c r="D15" s="1" t="s">
         <v>101</v>
       </c>
@@ -2575,8 +2719,8 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="46"/>
-      <c r="C16" s="46"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
       <c r="D16" s="1" t="s">
         <v>101</v>
       </c>
@@ -2591,10 +2735,10 @@
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="49">
+      <c r="B17" s="44">
         <v>46266</v>
       </c>
-      <c r="C17" s="51" t="s">
+      <c r="C17" s="46" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -2611,8 +2755,8 @@
       <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="49"/>
-      <c r="C18" s="49"/>
+      <c r="B18" s="44"/>
+      <c r="C18" s="44"/>
       <c r="D18" s="2" t="s">
         <v>103</v>
       </c>
@@ -2627,8 +2771,8 @@
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="49"/>
-      <c r="C19" s="49"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="44"/>
       <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
@@ -2643,8 +2787,8 @@
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="49"/>
-      <c r="C20" s="49"/>
+      <c r="B20" s="44"/>
+      <c r="C20" s="44"/>
       <c r="D20" s="2" t="s">
         <v>112</v>
       </c>
@@ -2659,10 +2803,10 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="46">
+      <c r="B21" s="45">
         <v>46267</v>
       </c>
-      <c r="C21" s="45" t="s">
+      <c r="C21" s="47" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -2679,8 +2823,8 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="46"/>
-      <c r="C22" s="46"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="45"/>
       <c r="D22" s="1" t="s">
         <v>102</v>
       </c>
@@ -2695,8 +2839,8 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="46"/>
-      <c r="C23" s="46"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="45"/>
       <c r="D23" s="1" t="s">
         <v>101</v>
       </c>
@@ -2711,8 +2855,8 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
+      <c r="B24" s="45"/>
+      <c r="C24" s="45"/>
       <c r="D24" s="1" t="s">
         <v>101</v>
       </c>
@@ -2727,8 +2871,8 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
+      <c r="B25" s="45"/>
+      <c r="C25" s="45"/>
       <c r="D25" s="1" t="s">
         <v>101</v>
       </c>
@@ -2743,13 +2887,13 @@
       <c r="A26" s="2">
         <v>24</v>
       </c>
-      <c r="B26" s="49">
+      <c r="B26" s="44">
         <v>46268</v>
       </c>
-      <c r="C26" s="51" t="s">
+      <c r="C26" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="55">
+      <c r="D26" s="43">
         <v>7</v>
       </c>
       <c r="E26" s="4" t="s">
@@ -2763,9 +2907,9 @@
       <c r="A27" s="2">
         <v>25</v>
       </c>
-      <c r="B27" s="49"/>
-      <c r="C27" s="49"/>
-      <c r="D27" s="49"/>
+      <c r="B27" s="44"/>
+      <c r="C27" s="44"/>
+      <c r="D27" s="44"/>
       <c r="E27" s="4" t="s">
         <v>36</v>
       </c>
@@ -2777,9 +2921,9 @@
       <c r="A28" s="2">
         <v>26</v>
       </c>
-      <c r="B28" s="49"/>
-      <c r="C28" s="49"/>
-      <c r="D28" s="49"/>
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
       <c r="E28" s="4" t="s">
         <v>37</v>
       </c>
@@ -2791,9 +2935,9 @@
       <c r="A29" s="2">
         <v>27</v>
       </c>
-      <c r="B29" s="49"/>
-      <c r="C29" s="49"/>
-      <c r="D29" s="49"/>
+      <c r="B29" s="44"/>
+      <c r="C29" s="44"/>
+      <c r="D29" s="44"/>
       <c r="E29" s="4" t="s">
         <v>38</v>
       </c>
@@ -2805,13 +2949,13 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="46">
+      <c r="B30" s="45">
         <v>46269</v>
       </c>
-      <c r="C30" s="45" t="s">
+      <c r="C30" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="54">
+      <c r="D30" s="48">
         <v>7</v>
       </c>
       <c r="E30" s="6" t="s">
@@ -2825,9 +2969,9 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="46"/>
-      <c r="C31" s="46"/>
-      <c r="D31" s="46"/>
+      <c r="B31" s="45"/>
+      <c r="C31" s="45"/>
+      <c r="D31" s="45"/>
       <c r="E31" s="6" t="s">
         <v>41</v>
       </c>
@@ -2839,9 +2983,9 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
+      <c r="B32" s="45"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
       <c r="E32" s="6" t="s">
         <v>42</v>
       </c>
@@ -2853,9 +2997,9 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="46"/>
-      <c r="C33" s="46"/>
-      <c r="D33" s="46"/>
+      <c r="B33" s="45"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
       <c r="E33" s="6" t="s">
         <v>43</v>
       </c>
@@ -2867,13 +3011,13 @@
       <c r="A34" s="2">
         <v>32</v>
       </c>
-      <c r="B34" s="49">
+      <c r="B34" s="44">
         <v>46272</v>
       </c>
-      <c r="C34" s="51" t="s">
+      <c r="C34" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="55">
+      <c r="D34" s="43">
         <v>8</v>
       </c>
       <c r="E34" s="4" t="s">
@@ -2887,9 +3031,9 @@
       <c r="A35" s="2">
         <v>33</v>
       </c>
-      <c r="B35" s="49"/>
-      <c r="C35" s="49"/>
-      <c r="D35" s="49"/>
+      <c r="B35" s="44"/>
+      <c r="C35" s="44"/>
+      <c r="D35" s="44"/>
       <c r="E35" s="4" t="s">
         <v>46</v>
       </c>
@@ -2901,9 +3045,9 @@
       <c r="A36" s="2">
         <v>34</v>
       </c>
-      <c r="B36" s="49"/>
-      <c r="C36" s="49"/>
-      <c r="D36" s="49"/>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
       <c r="E36" s="4" t="s">
         <v>47</v>
       </c>
@@ -2915,9 +3059,9 @@
       <c r="A37" s="2">
         <v>35</v>
       </c>
-      <c r="B37" s="49"/>
-      <c r="C37" s="49"/>
-      <c r="D37" s="49"/>
+      <c r="B37" s="44"/>
+      <c r="C37" s="44"/>
+      <c r="D37" s="44"/>
       <c r="E37" s="4" t="s">
         <v>48</v>
       </c>
@@ -2929,9 +3073,9 @@
       <c r="A38" s="2">
         <v>36</v>
       </c>
-      <c r="B38" s="49"/>
-      <c r="C38" s="49"/>
-      <c r="D38" s="49"/>
+      <c r="B38" s="44"/>
+      <c r="C38" s="44"/>
+      <c r="D38" s="44"/>
       <c r="E38" s="4" t="s">
         <v>49</v>
       </c>
@@ -2943,13 +3087,13 @@
       <c r="A39" s="1">
         <v>37</v>
       </c>
-      <c r="B39" s="46">
+      <c r="B39" s="45">
         <v>46273</v>
       </c>
-      <c r="C39" s="45" t="s">
+      <c r="C39" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="D39" s="54">
+      <c r="D39" s="48">
         <v>6</v>
       </c>
       <c r="E39" s="6" t="s">
@@ -2963,9 +3107,9 @@
       <c r="A40" s="1">
         <v>38</v>
       </c>
-      <c r="B40" s="46"/>
-      <c r="C40" s="46"/>
-      <c r="D40" s="46"/>
+      <c r="B40" s="45"/>
+      <c r="C40" s="45"/>
+      <c r="D40" s="45"/>
       <c r="E40" s="6" t="s">
         <v>51</v>
       </c>
@@ -2977,9 +3121,9 @@
       <c r="A41" s="1">
         <v>39</v>
       </c>
-      <c r="B41" s="46"/>
-      <c r="C41" s="46"/>
-      <c r="D41" s="46"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="45"/>
+      <c r="D41" s="45"/>
       <c r="E41" s="6" t="s">
         <v>52</v>
       </c>
@@ -2991,9 +3135,9 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" s="46"/>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
+      <c r="B42" s="45"/>
+      <c r="C42" s="45"/>
+      <c r="D42" s="45"/>
       <c r="E42" s="6" t="s">
         <v>53</v>
       </c>
@@ -3005,9 +3149,9 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" s="46"/>
-      <c r="C43" s="46"/>
-      <c r="D43" s="46"/>
+      <c r="B43" s="45"/>
+      <c r="C43" s="45"/>
+      <c r="D43" s="45"/>
       <c r="E43" s="6" t="s">
         <v>54</v>
       </c>
@@ -3019,9 +3163,9 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" s="46"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="46"/>
+      <c r="B44" s="45"/>
+      <c r="C44" s="45"/>
+      <c r="D44" s="45"/>
       <c r="E44" s="6" t="s">
         <v>55</v>
       </c>
@@ -3033,9 +3177,9 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" s="46"/>
-      <c r="C45" s="46"/>
-      <c r="D45" s="46"/>
+      <c r="B45" s="45"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
       <c r="E45" s="6" t="s">
         <v>56</v>
       </c>
@@ -3047,10 +3191,10 @@
       <c r="A46" s="2">
         <v>44</v>
       </c>
-      <c r="B46" s="49">
+      <c r="B46" s="44">
         <v>46274</v>
       </c>
-      <c r="C46" s="51" t="s">
+      <c r="C46" s="46" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="2" t="s">
@@ -3067,8 +3211,8 @@
       <c r="A47" s="2">
         <v>45</v>
       </c>
-      <c r="B47" s="49"/>
-      <c r="C47" s="49"/>
+      <c r="B47" s="44"/>
+      <c r="C47" s="44"/>
       <c r="D47" s="2" t="s">
         <v>99</v>
       </c>
@@ -3081,8 +3225,8 @@
     </row>
     <row r="48" spans="1:6" ht="34.5" customHeight="1">
       <c r="A48" s="2"/>
-      <c r="B48" s="49"/>
-      <c r="C48" s="49"/>
+      <c r="B48" s="44"/>
+      <c r="C48" s="44"/>
       <c r="D48" s="2" t="s">
         <v>102</v>
       </c>
@@ -3095,8 +3239,8 @@
       <c r="A49" s="2">
         <v>46</v>
       </c>
-      <c r="B49" s="49"/>
-      <c r="C49" s="49"/>
+      <c r="B49" s="44"/>
+      <c r="C49" s="44"/>
       <c r="D49" s="2" t="s">
         <v>100</v>
       </c>
@@ -3108,13 +3252,13 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A50" s="45">
+      <c r="A50" s="47">
         <v>47</v>
       </c>
-      <c r="B50" s="46">
+      <c r="B50" s="45">
         <v>46275</v>
       </c>
-      <c r="C50" s="45" t="s">
+      <c r="C50" s="47" t="s">
         <v>14</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -3128,9 +3272,9 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A51" s="45"/>
-      <c r="B51" s="45"/>
-      <c r="C51" s="45"/>
+      <c r="A51" s="47"/>
+      <c r="B51" s="47"/>
+      <c r="C51" s="47"/>
       <c r="D51" s="1" t="s">
         <v>100</v>
       </c>
@@ -3145,10 +3289,10 @@
       <c r="A52" s="2">
         <v>49</v>
       </c>
-      <c r="B52" s="49">
+      <c r="B52" s="44">
         <v>46276</v>
       </c>
-      <c r="C52" s="51" t="s">
+      <c r="C52" s="46" t="s">
         <v>39</v>
       </c>
       <c r="D52" s="2" t="s">
@@ -3165,8 +3309,8 @@
       <c r="A53" s="2">
         <v>50</v>
       </c>
-      <c r="B53" s="49"/>
-      <c r="C53" s="49"/>
+      <c r="B53" s="44"/>
+      <c r="C53" s="44"/>
       <c r="D53" s="2" t="s">
         <v>105</v>
       </c>
@@ -3181,8 +3325,8 @@
       <c r="A54" s="2">
         <v>51</v>
       </c>
-      <c r="B54" s="49"/>
-      <c r="C54" s="49"/>
+      <c r="B54" s="44"/>
+      <c r="C54" s="44"/>
       <c r="D54" s="2" t="s">
         <v>107</v>
       </c>
@@ -3197,8 +3341,8 @@
       <c r="A55" s="2">
         <v>52</v>
       </c>
-      <c r="B55" s="49"/>
-      <c r="C55" s="49"/>
+      <c r="B55" s="44"/>
+      <c r="C55" s="44"/>
       <c r="D55" s="2" t="s">
         <v>99</v>
       </c>
@@ -3211,8 +3355,8 @@
     </row>
     <row r="56" spans="1:6" ht="34.5" customHeight="1">
       <c r="A56" s="2"/>
-      <c r="B56" s="49"/>
-      <c r="C56" s="49"/>
+      <c r="B56" s="44"/>
+      <c r="C56" s="44"/>
       <c r="D56" s="2" t="s">
         <v>102</v>
       </c>
@@ -3225,8 +3369,8 @@
       <c r="A57" s="2">
         <v>53</v>
       </c>
-      <c r="B57" s="49"/>
-      <c r="C57" s="49"/>
+      <c r="B57" s="44"/>
+      <c r="C57" s="44"/>
       <c r="D57" s="2" t="s">
         <v>105</v>
       </c>
@@ -3241,10 +3385,10 @@
       <c r="A58" s="1">
         <v>54</v>
       </c>
-      <c r="B58" s="46">
+      <c r="B58" s="45">
         <v>46280</v>
       </c>
-      <c r="C58" s="45" t="s">
+      <c r="C58" s="47" t="s">
         <v>24</v>
       </c>
       <c r="D58" s="1" t="s">
@@ -3261,8 +3405,8 @@
       <c r="A59" s="1">
         <v>55</v>
       </c>
-      <c r="B59" s="46"/>
-      <c r="C59" s="46"/>
+      <c r="B59" s="45"/>
+      <c r="C59" s="45"/>
       <c r="D59" s="1" t="s">
         <v>102</v>
       </c>
@@ -3277,8 +3421,8 @@
       <c r="A60" s="1">
         <v>56</v>
       </c>
-      <c r="B60" s="46"/>
-      <c r="C60" s="46"/>
+      <c r="B60" s="45"/>
+      <c r="C60" s="45"/>
       <c r="D60" s="1" t="s">
         <v>105</v>
       </c>
@@ -3293,8 +3437,8 @@
       <c r="A61" s="1">
         <v>57</v>
       </c>
-      <c r="B61" s="46"/>
-      <c r="C61" s="46"/>
+      <c r="B61" s="45"/>
+      <c r="C61" s="45"/>
       <c r="D61" s="1" t="s">
         <v>106</v>
       </c>
@@ -3309,10 +3453,10 @@
       <c r="A62" s="2">
         <v>58</v>
       </c>
-      <c r="B62" s="49">
+      <c r="B62" s="44">
         <v>46281</v>
       </c>
-      <c r="C62" s="51" t="s">
+      <c r="C62" s="46" t="s">
         <v>7</v>
       </c>
       <c r="D62" s="2" t="s">
@@ -3329,8 +3473,8 @@
       <c r="A63" s="2">
         <v>59</v>
       </c>
-      <c r="B63" s="49"/>
-      <c r="C63" s="49"/>
+      <c r="B63" s="44"/>
+      <c r="C63" s="44"/>
       <c r="D63" s="2" t="s">
         <v>102</v>
       </c>
@@ -3345,8 +3489,8 @@
       <c r="A64" s="2">
         <v>60</v>
       </c>
-      <c r="B64" s="49"/>
-      <c r="C64" s="49"/>
+      <c r="B64" s="44"/>
+      <c r="C64" s="44"/>
       <c r="D64" s="2" t="s">
         <v>101</v>
       </c>
@@ -3361,8 +3505,8 @@
       <c r="A65" s="2">
         <v>61</v>
       </c>
-      <c r="B65" s="49"/>
-      <c r="C65" s="49"/>
+      <c r="B65" s="44"/>
+      <c r="C65" s="44"/>
       <c r="D65" s="2" t="s">
         <v>101</v>
       </c>
@@ -3377,8 +3521,8 @@
       <c r="A66" s="2">
         <v>62</v>
       </c>
-      <c r="B66" s="49"/>
-      <c r="C66" s="49"/>
+      <c r="B66" s="44"/>
+      <c r="C66" s="44"/>
       <c r="D66" s="2" t="s">
         <v>102</v>
       </c>
@@ -3393,10 +3537,10 @@
       <c r="A67" s="1">
         <v>63</v>
       </c>
-      <c r="B67" s="46">
+      <c r="B67" s="45">
         <v>46282</v>
       </c>
-      <c r="C67" s="45" t="s">
+      <c r="C67" s="47" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -3413,8 +3557,8 @@
       <c r="A68" s="1">
         <v>64</v>
       </c>
-      <c r="B68" s="46"/>
-      <c r="C68" s="46"/>
+      <c r="B68" s="45"/>
+      <c r="C68" s="45"/>
       <c r="D68" s="1" t="s">
         <v>105</v>
       </c>
@@ -3429,8 +3573,8 @@
       <c r="A69" s="1">
         <v>65</v>
       </c>
-      <c r="B69" s="46"/>
-      <c r="C69" s="46"/>
+      <c r="B69" s="45"/>
+      <c r="C69" s="45"/>
       <c r="D69" s="1" t="s">
         <v>102</v>
       </c>
@@ -3445,8 +3589,8 @@
       <c r="A70" s="1">
         <v>66</v>
       </c>
-      <c r="B70" s="46"/>
-      <c r="C70" s="46"/>
+      <c r="B70" s="45"/>
+      <c r="C70" s="45"/>
       <c r="D70" s="1" t="s">
         <v>104</v>
       </c>
@@ -3461,13 +3605,13 @@
       <c r="A71" s="2">
         <v>67</v>
       </c>
-      <c r="B71" s="49">
+      <c r="B71" s="44">
         <v>46283</v>
       </c>
-      <c r="C71" s="51" t="s">
+      <c r="C71" s="46" t="s">
         <v>39</v>
       </c>
-      <c r="D71" s="55">
+      <c r="D71" s="43">
         <v>7</v>
       </c>
       <c r="E71" s="4" t="s">
@@ -3481,9 +3625,9 @@
       <c r="A72" s="2">
         <v>68</v>
       </c>
-      <c r="B72" s="49"/>
-      <c r="C72" s="49"/>
-      <c r="D72" s="49"/>
+      <c r="B72" s="44"/>
+      <c r="C72" s="44"/>
+      <c r="D72" s="44"/>
       <c r="E72" s="4" t="s">
         <v>82</v>
       </c>
@@ -3495,9 +3639,9 @@
       <c r="A73" s="2">
         <v>69</v>
       </c>
-      <c r="B73" s="49"/>
-      <c r="C73" s="49"/>
-      <c r="D73" s="49"/>
+      <c r="B73" s="44"/>
+      <c r="C73" s="44"/>
+      <c r="D73" s="44"/>
       <c r="E73" s="4" t="s">
         <v>83</v>
       </c>
@@ -3509,9 +3653,9 @@
       <c r="A74" s="2">
         <v>70</v>
       </c>
-      <c r="B74" s="49"/>
-      <c r="C74" s="49"/>
-      <c r="D74" s="49"/>
+      <c r="B74" s="44"/>
+      <c r="C74" s="44"/>
+      <c r="D74" s="44"/>
       <c r="E74" s="4" t="s">
         <v>84</v>
       </c>
@@ -3523,9 +3667,9 @@
       <c r="A75" s="2">
         <v>71</v>
       </c>
-      <c r="B75" s="49"/>
-      <c r="C75" s="49"/>
-      <c r="D75" s="49"/>
+      <c r="B75" s="44"/>
+      <c r="C75" s="44"/>
+      <c r="D75" s="44"/>
       <c r="E75" s="4" t="s">
         <v>85</v>
       </c>
@@ -3537,9 +3681,9 @@
       <c r="A76" s="2">
         <v>72</v>
       </c>
-      <c r="B76" s="49"/>
-      <c r="C76" s="49"/>
-      <c r="D76" s="49"/>
+      <c r="B76" s="44"/>
+      <c r="C76" s="44"/>
+      <c r="D76" s="44"/>
       <c r="E76" s="4" t="s">
         <v>86</v>
       </c>
@@ -3551,9 +3695,9 @@
       <c r="A77" s="2">
         <v>73</v>
       </c>
-      <c r="B77" s="49"/>
-      <c r="C77" s="49"/>
-      <c r="D77" s="49"/>
+      <c r="B77" s="44"/>
+      <c r="C77" s="44"/>
+      <c r="D77" s="44"/>
       <c r="E77" s="4" t="s">
         <v>87</v>
       </c>
@@ -3565,10 +3709,10 @@
       <c r="A78" s="1">
         <v>74</v>
       </c>
-      <c r="B78" s="46">
+      <c r="B78" s="45">
         <v>46286</v>
       </c>
-      <c r="C78" s="45" t="s">
+      <c r="C78" s="47" t="s">
         <v>44</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -3585,8 +3729,8 @@
       <c r="A79" s="1">
         <v>75</v>
       </c>
-      <c r="B79" s="46"/>
-      <c r="C79" s="46"/>
+      <c r="B79" s="45"/>
+      <c r="C79" s="45"/>
       <c r="D79" s="1" t="s">
         <v>102</v>
       </c>
@@ -3601,8 +3745,8 @@
       <c r="A80" s="1">
         <v>76</v>
       </c>
-      <c r="B80" s="46"/>
-      <c r="C80" s="46"/>
+      <c r="B80" s="45"/>
+      <c r="C80" s="45"/>
       <c r="D80" s="1" t="s">
         <v>103</v>
       </c>
@@ -3617,8 +3761,8 @@
       <c r="A81" s="1">
         <v>77</v>
       </c>
-      <c r="B81" s="46"/>
-      <c r="C81" s="46"/>
+      <c r="B81" s="45"/>
+      <c r="C81" s="45"/>
       <c r="D81" s="1" t="s">
         <v>102</v>
       </c>
@@ -3633,8 +3777,8 @@
       <c r="A82" s="1">
         <v>78</v>
       </c>
-      <c r="B82" s="46"/>
-      <c r="C82" s="46"/>
+      <c r="B82" s="45"/>
+      <c r="C82" s="45"/>
       <c r="D82" s="1" t="s">
         <v>101</v>
       </c>
@@ -3649,8 +3793,8 @@
       <c r="A83" s="1">
         <v>79</v>
       </c>
-      <c r="B83" s="46"/>
-      <c r="C83" s="46"/>
+      <c r="B83" s="45"/>
+      <c r="C83" s="45"/>
       <c r="D83" s="1" t="s">
         <v>102</v>
       </c>
@@ -3665,10 +3809,10 @@
       <c r="A84" s="2">
         <v>80</v>
       </c>
-      <c r="B84" s="49">
+      <c r="B84" s="44">
         <v>46287</v>
       </c>
-      <c r="C84" s="51" t="s">
+      <c r="C84" s="46" t="s">
         <v>24</v>
       </c>
       <c r="D84" s="2" t="s">
@@ -3685,8 +3829,8 @@
       <c r="A85" s="2">
         <v>81</v>
       </c>
-      <c r="B85" s="49"/>
-      <c r="C85" s="49"/>
+      <c r="B85" s="44"/>
+      <c r="C85" s="44"/>
       <c r="D85" s="2" t="s">
         <v>99</v>
       </c>
@@ -3701,8 +3845,8 @@
       <c r="A86" s="2">
         <v>82</v>
       </c>
-      <c r="B86" s="49"/>
-      <c r="C86" s="49"/>
+      <c r="B86" s="44"/>
+      <c r="C86" s="44"/>
       <c r="D86" s="2" t="s">
         <v>100</v>
       </c>
@@ -3717,8 +3861,8 @@
       <c r="A87" s="2">
         <v>83</v>
       </c>
-      <c r="B87" s="49"/>
-      <c r="C87" s="49"/>
+      <c r="B87" s="44"/>
+      <c r="C87" s="44"/>
       <c r="D87" s="2" t="s">
         <v>101</v>
       </c>
@@ -3731,8 +3875,8 @@
     </row>
     <row r="88" spans="1:6" ht="20.25" customHeight="1">
       <c r="A88" s="2"/>
-      <c r="B88" s="49"/>
-      <c r="C88" s="49"/>
+      <c r="B88" s="44"/>
+      <c r="C88" s="44"/>
       <c r="D88" s="2" t="s">
         <v>101</v>
       </c>
@@ -3745,8 +3889,8 @@
       <c r="A89" s="9">
         <v>84</v>
       </c>
-      <c r="B89" s="50"/>
-      <c r="C89" s="50"/>
+      <c r="B89" s="58"/>
+      <c r="C89" s="58"/>
       <c r="D89" s="9" t="s">
         <v>101</v>
       </c>
@@ -3761,10 +3905,10 @@
       <c r="A90" s="12">
         <v>85</v>
       </c>
-      <c r="B90" s="48">
+      <c r="B90" s="57">
         <v>46288</v>
       </c>
-      <c r="C90" s="47" t="s">
+      <c r="C90" s="56" t="s">
         <v>7</v>
       </c>
       <c r="D90" s="12" t="s">
@@ -3781,8 +3925,8 @@
       <c r="A91" s="15">
         <v>86</v>
       </c>
-      <c r="B91" s="48"/>
-      <c r="C91" s="47"/>
+      <c r="B91" s="57"/>
+      <c r="C91" s="56"/>
       <c r="D91" s="15" t="s">
         <v>101</v>
       </c>
@@ -3797,8 +3941,8 @@
       <c r="A92" s="18">
         <v>87</v>
       </c>
-      <c r="B92" s="48"/>
-      <c r="C92" s="47"/>
+      <c r="B92" s="57"/>
+      <c r="C92" s="56"/>
       <c r="D92" s="15" t="s">
         <v>117</v>
       </c>
@@ -3813,8 +3957,8 @@
       <c r="A93" s="19">
         <v>88</v>
       </c>
-      <c r="B93" s="48"/>
-      <c r="C93" s="47"/>
+      <c r="B93" s="57"/>
+      <c r="C93" s="56"/>
       <c r="D93" s="15" t="s">
         <v>100</v>
       </c>
@@ -3829,8 +3973,8 @@
       <c r="A94" s="20">
         <v>89</v>
       </c>
-      <c r="B94" s="48"/>
-      <c r="C94" s="47"/>
+      <c r="B94" s="57"/>
+      <c r="C94" s="56"/>
       <c r="D94" s="15" t="s">
         <v>101</v>
       </c>
@@ -3845,605 +3989,769 @@
       <c r="A95" s="20">
         <v>90</v>
       </c>
-      <c r="B95" s="48"/>
+      <c r="B95" s="57"/>
       <c r="C95" s="17"/>
       <c r="D95" s="17"/>
       <c r="E95" s="17"/>
       <c r="F95" s="17"/>
     </row>
     <row r="96" spans="1:6">
-      <c r="A96" s="24">
+      <c r="A96" s="23">
         <v>91</v>
       </c>
-      <c r="B96" s="52">
+      <c r="B96" s="59">
         <v>46289</v>
       </c>
-      <c r="C96" s="53" t="s">
+      <c r="C96" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="D96" s="25" t="s">
+      <c r="D96" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E96" s="23" t="s">
+      <c r="E96" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="F96" s="23"/>
+      <c r="F96" s="22"/>
     </row>
     <row r="97" spans="1:6" ht="60">
-      <c r="A97" s="24">
+      <c r="A97" s="23">
         <v>92</v>
       </c>
-      <c r="B97" s="52"/>
-      <c r="C97" s="53"/>
-      <c r="D97" s="25" t="s">
+      <c r="B97" s="59"/>
+      <c r="C97" s="60"/>
+      <c r="D97" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E97" s="26" t="s">
+      <c r="E97" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="F97" s="23"/>
+      <c r="F97" s="22"/>
     </row>
     <row r="98" spans="1:6" ht="60">
-      <c r="A98" s="24">
+      <c r="A98" s="23">
         <v>93</v>
       </c>
-      <c r="B98" s="52"/>
-      <c r="C98" s="53"/>
-      <c r="D98" s="25" t="s">
+      <c r="B98" s="59"/>
+      <c r="C98" s="60"/>
+      <c r="D98" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E98" s="27" t="s">
+      <c r="E98" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="F98" s="23"/>
+      <c r="F98" s="22"/>
     </row>
     <row r="99" spans="1:6" ht="30">
-      <c r="A99" s="24">
+      <c r="A99" s="23">
         <v>94</v>
       </c>
-      <c r="B99" s="52"/>
-      <c r="C99" s="53"/>
-      <c r="D99" s="25" t="s">
+      <c r="B99" s="59"/>
+      <c r="C99" s="60"/>
+      <c r="D99" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E99" s="28" t="s">
+      <c r="E99" s="27" t="s">
         <v>123</v>
       </c>
-      <c r="F99" s="23"/>
+      <c r="F99" s="22"/>
     </row>
     <row r="100" spans="1:6">
-      <c r="A100" s="24">
+      <c r="A100" s="23">
         <v>95</v>
       </c>
-      <c r="B100" s="52"/>
-      <c r="C100" s="53"/>
-      <c r="D100" s="25" t="s">
+      <c r="B100" s="59"/>
+      <c r="C100" s="60"/>
+      <c r="D100" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="E100" s="29" t="s">
+      <c r="E100" s="28" t="s">
         <v>124</v>
       </c>
-      <c r="F100" s="23"/>
+      <c r="F100" s="22"/>
     </row>
     <row r="101" spans="1:6" ht="30">
-      <c r="A101" s="24">
+      <c r="A101" s="23">
         <v>96</v>
       </c>
-      <c r="B101" s="52"/>
-      <c r="C101" s="53"/>
-      <c r="D101" s="25" t="s">
+      <c r="B101" s="59"/>
+      <c r="C101" s="60"/>
+      <c r="D101" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E101" s="26" t="s">
+      <c r="E101" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="F101" s="23"/>
+      <c r="F101" s="22"/>
     </row>
     <row r="102" spans="1:6" ht="45">
-      <c r="A102" s="24">
+      <c r="A102" s="23">
         <v>97</v>
       </c>
-      <c r="B102" s="52"/>
-      <c r="C102" s="53"/>
-      <c r="D102" s="25" t="s">
+      <c r="B102" s="59"/>
+      <c r="C102" s="60"/>
+      <c r="D102" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="E102" s="28" t="s">
+      <c r="E102" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="F102" s="23"/>
+      <c r="F102" s="22"/>
     </row>
     <row r="103" spans="1:6">
-      <c r="A103" s="24">
+      <c r="A103" s="23">
         <v>98</v>
       </c>
-      <c r="B103" s="52"/>
-      <c r="C103" s="53"/>
-      <c r="D103" s="23"/>
-      <c r="E103" s="23"/>
-      <c r="F103" s="23"/>
+      <c r="B103" s="59"/>
+      <c r="C103" s="60"/>
+      <c r="D103" s="22"/>
+      <c r="E103" s="22"/>
+      <c r="F103" s="22"/>
     </row>
     <row r="104" spans="1:6">
-      <c r="A104" s="24">
+      <c r="A104" s="23">
         <v>99</v>
       </c>
-      <c r="B104" s="52"/>
-      <c r="C104" s="53"/>
-      <c r="D104" s="25" t="s">
+      <c r="B104" s="59"/>
+      <c r="C104" s="60"/>
+      <c r="D104" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="E104" s="30" t="s">
+      <c r="E104" s="29" t="s">
         <v>127</v>
       </c>
-      <c r="F104" s="23"/>
+      <c r="F104" s="22"/>
     </row>
     <row r="105" spans="1:6">
-      <c r="A105" s="24">
+      <c r="A105" s="23">
         <v>100</v>
       </c>
-      <c r="B105" s="52"/>
-      <c r="C105" s="53"/>
-      <c r="D105" s="25" t="s">
+      <c r="B105" s="59"/>
+      <c r="C105" s="60"/>
+      <c r="D105" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="E105" s="23" t="s">
+      <c r="E105" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="F105" s="23"/>
+      <c r="F105" s="22"/>
     </row>
     <row r="106" spans="1:6">
-      <c r="A106" s="24">
+      <c r="A106" s="23">
         <v>101</v>
       </c>
-      <c r="B106" s="52"/>
-      <c r="C106" s="53"/>
-      <c r="D106" s="25" t="s">
+      <c r="B106" s="59"/>
+      <c r="C106" s="60"/>
+      <c r="D106" s="24" t="s">
         <v>130</v>
       </c>
-      <c r="E106" s="23" t="s">
+      <c r="E106" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="F106" s="23"/>
+      <c r="F106" s="22"/>
     </row>
     <row r="107" spans="1:6" ht="45">
-      <c r="A107" s="24">
+      <c r="A107" s="23">
         <v>102</v>
       </c>
-      <c r="B107" s="52"/>
-      <c r="C107" s="53"/>
-      <c r="D107" s="25" t="s">
+      <c r="B107" s="59"/>
+      <c r="C107" s="60"/>
+      <c r="D107" s="24" t="s">
         <v>101</v>
       </c>
-      <c r="E107" s="27" t="s">
+      <c r="E107" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="F107" s="23"/>
+      <c r="F107" s="22"/>
     </row>
     <row r="108" spans="1:6" ht="45">
-      <c r="A108" s="24">
+      <c r="A108" s="23">
         <v>103</v>
       </c>
-      <c r="B108" s="52"/>
-      <c r="C108" s="53"/>
-      <c r="D108" s="25" t="s">
+      <c r="B108" s="59"/>
+      <c r="C108" s="60"/>
+      <c r="D108" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="E108" s="27" t="s">
+      <c r="E108" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="F108" s="23"/>
+      <c r="F108" s="22"/>
     </row>
     <row r="109" spans="1:6">
-      <c r="A109" s="24">
+      <c r="A109" s="23">
         <v>104</v>
       </c>
-      <c r="B109" s="52"/>
-      <c r="C109" s="53"/>
-      <c r="D109" s="25" t="s">
+      <c r="B109" s="59"/>
+      <c r="C109" s="60"/>
+      <c r="D109" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="E109" s="23" t="s">
+      <c r="E109" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="F109" s="23"/>
+      <c r="F109" s="22"/>
     </row>
     <row r="110" spans="1:6" ht="45">
-      <c r="A110" s="24">
+      <c r="A110" s="23">
         <v>105</v>
       </c>
-      <c r="B110" s="39">
+      <c r="B110" s="50">
         <v>46290</v>
       </c>
-      <c r="C110" s="42" t="s">
+      <c r="C110" s="53" t="s">
         <v>39</v>
       </c>
       <c r="D110" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="E110" s="33" t="s">
+      <c r="E110" s="32" t="s">
         <v>135</v>
       </c>
-      <c r="F110" s="32"/>
+      <c r="F110" s="31"/>
     </row>
     <row r="111" spans="1:6" ht="45">
-      <c r="A111" s="32"/>
-      <c r="B111" s="40"/>
-      <c r="C111" s="43"/>
-      <c r="D111" s="25" t="s">
+      <c r="A111" s="31"/>
+      <c r="B111" s="51"/>
+      <c r="C111" s="54"/>
+      <c r="D111" s="24" t="s">
         <v>137</v>
       </c>
-      <c r="E111" s="33" t="s">
+      <c r="E111" s="32" t="s">
         <v>136</v>
       </c>
-      <c r="F111" s="32"/>
+      <c r="F111" s="31"/>
     </row>
     <row r="112" spans="1:6">
-      <c r="A112" s="32"/>
-      <c r="B112" s="40"/>
-      <c r="C112" s="43"/>
-      <c r="D112" s="32"/>
-      <c r="E112" s="32"/>
-      <c r="F112" s="32"/>
+      <c r="A112" s="31"/>
+      <c r="B112" s="51"/>
+      <c r="C112" s="54"/>
+      <c r="D112" s="31"/>
+      <c r="E112" s="31"/>
+      <c r="F112" s="31"/>
     </row>
     <row r="113" spans="1:6" ht="45">
-      <c r="A113" s="32"/>
-      <c r="B113" s="40"/>
-      <c r="C113" s="43"/>
-      <c r="D113" s="32" t="s">
+      <c r="A113" s="31"/>
+      <c r="B113" s="51"/>
+      <c r="C113" s="54"/>
+      <c r="D113" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="E113" s="33" t="s">
+      <c r="E113" s="32" t="s">
         <v>138</v>
       </c>
-      <c r="F113" s="32"/>
+      <c r="F113" s="31"/>
     </row>
     <row r="114" spans="1:6" ht="60">
-      <c r="A114" s="32"/>
-      <c r="B114" s="40"/>
-      <c r="C114" s="43"/>
-      <c r="D114" s="32" t="s">
+      <c r="A114" s="31"/>
+      <c r="B114" s="51"/>
+      <c r="C114" s="54"/>
+      <c r="D114" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="E114" s="34" t="s">
+      <c r="E114" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="F114" s="32"/>
+      <c r="F114" s="31"/>
     </row>
     <row r="115" spans="1:6" ht="75">
-      <c r="A115" s="32"/>
-      <c r="B115" s="40"/>
-      <c r="C115" s="43"/>
-      <c r="D115" s="32" t="s">
+      <c r="A115" s="31"/>
+      <c r="B115" s="51"/>
+      <c r="C115" s="54"/>
+      <c r="D115" s="31" t="s">
         <v>140</v>
       </c>
-      <c r="E115" s="33" t="s">
+      <c r="E115" s="32" t="s">
         <v>142</v>
       </c>
-      <c r="F115" s="32" t="s">
+      <c r="F115" s="31" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="116" spans="1:6">
-      <c r="A116" s="32"/>
-      <c r="B116" s="40"/>
-      <c r="C116" s="43"/>
-      <c r="D116" s="32" t="s">
+      <c r="A116" s="31"/>
+      <c r="B116" s="51"/>
+      <c r="C116" s="54"/>
+      <c r="D116" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="E116" s="33" t="s">
+      <c r="E116" s="32" t="s">
         <v>141</v>
       </c>
-      <c r="F116" s="32"/>
+      <c r="F116" s="31"/>
     </row>
     <row r="117" spans="1:6" ht="45">
-      <c r="A117" s="32"/>
-      <c r="B117" s="40"/>
-      <c r="C117" s="43"/>
-      <c r="D117" s="32"/>
-      <c r="E117" s="33" t="s">
+      <c r="A117" s="31"/>
+      <c r="B117" s="51"/>
+      <c r="C117" s="54"/>
+      <c r="D117" s="31"/>
+      <c r="E117" s="32" t="s">
         <v>147</v>
       </c>
-      <c r="F117" s="32" t="s">
+      <c r="F117" s="31" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="118" spans="1:6">
-      <c r="A118" s="32"/>
-      <c r="B118" s="40"/>
-      <c r="C118" s="43"/>
-      <c r="D118" s="32"/>
-      <c r="E118" s="32"/>
-      <c r="F118" s="32"/>
+      <c r="A118" s="31"/>
+      <c r="B118" s="51"/>
+      <c r="C118" s="54"/>
+      <c r="D118" s="31"/>
+      <c r="E118" s="31"/>
+      <c r="F118" s="31"/>
     </row>
     <row r="119" spans="1:6" ht="30">
-      <c r="A119" s="32"/>
-      <c r="B119" s="40"/>
-      <c r="C119" s="43"/>
-      <c r="D119" s="32"/>
-      <c r="E119" s="34" t="s">
+      <c r="A119" s="31"/>
+      <c r="B119" s="51"/>
+      <c r="C119" s="54"/>
+      <c r="D119" s="31"/>
+      <c r="E119" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="F119" s="32" t="s">
+      <c r="F119" s="31" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="75">
-      <c r="A120" s="32"/>
-      <c r="B120" s="40"/>
-      <c r="C120" s="43"/>
-      <c r="D120" s="32" t="s">
+      <c r="A120" s="31"/>
+      <c r="B120" s="51"/>
+      <c r="C120" s="54"/>
+      <c r="D120" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="E120" s="33" t="s">
+      <c r="E120" s="32" t="s">
         <v>146</v>
       </c>
-      <c r="F120" s="33" t="s">
+      <c r="F120" s="32" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="45">
-      <c r="A121" s="32"/>
-      <c r="B121" s="41"/>
-      <c r="C121" s="44"/>
-      <c r="D121" s="32" t="s">
+      <c r="A121" s="31"/>
+      <c r="B121" s="52"/>
+      <c r="C121" s="55"/>
+      <c r="D121" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="E121" s="33" t="s">
+      <c r="E121" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="F121" s="32"/>
+      <c r="F121" s="31"/>
     </row>
     <row r="122" spans="1:6" ht="30">
-      <c r="A122" s="35"/>
-      <c r="B122" s="57">
+      <c r="A122" s="34"/>
+      <c r="B122" s="37">
         <v>46293</v>
       </c>
-      <c r="C122" s="60" t="s">
+      <c r="C122" s="40" t="s">
         <v>44</v>
       </c>
-      <c r="D122" s="35" t="s">
+      <c r="D122" s="34" t="s">
         <v>152</v>
       </c>
-      <c r="E122" s="36" t="s">
+      <c r="E122" s="35" t="s">
         <v>151</v>
       </c>
-      <c r="F122" s="35"/>
+      <c r="F122" s="34"/>
     </row>
     <row r="123" spans="1:6" ht="75">
-      <c r="A123" s="35"/>
-      <c r="B123" s="58"/>
-      <c r="C123" s="61"/>
-      <c r="D123" s="35" t="s">
+      <c r="A123" s="34"/>
+      <c r="B123" s="38"/>
+      <c r="C123" s="41"/>
+      <c r="D123" s="34" t="s">
         <v>157</v>
       </c>
-      <c r="E123" s="37" t="s">
+      <c r="E123" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="F123" s="35"/>
+      <c r="F123" s="34"/>
     </row>
     <row r="124" spans="1:6">
-      <c r="A124" s="35"/>
-      <c r="B124" s="58"/>
-      <c r="C124" s="61"/>
-      <c r="D124" s="35" t="s">
+      <c r="A124" s="34"/>
+      <c r="B124" s="38"/>
+      <c r="C124" s="41"/>
+      <c r="D124" s="34" t="s">
         <v>102</v>
       </c>
-      <c r="E124" s="37" t="s">
+      <c r="E124" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="F124" s="35"/>
+      <c r="F124" s="34"/>
     </row>
     <row r="125" spans="1:6">
-      <c r="A125" s="35"/>
-      <c r="B125" s="58"/>
-      <c r="C125" s="61"/>
-      <c r="D125" s="35" t="s">
+      <c r="A125" s="34"/>
+      <c r="B125" s="38"/>
+      <c r="C125" s="41"/>
+      <c r="D125" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="E125" s="37" t="s">
+      <c r="E125" s="36" t="s">
         <v>154</v>
       </c>
-      <c r="F125" s="35"/>
+      <c r="F125" s="34"/>
     </row>
     <row r="126" spans="1:6">
-      <c r="A126" s="35"/>
-      <c r="B126" s="58"/>
-      <c r="C126" s="61"/>
-      <c r="D126" s="35" t="s">
+      <c r="A126" s="34"/>
+      <c r="B126" s="38"/>
+      <c r="C126" s="41"/>
+      <c r="D126" s="34" t="s">
         <v>117</v>
       </c>
-      <c r="E126" s="37" t="s">
+      <c r="E126" s="36" t="s">
         <v>156</v>
       </c>
-      <c r="F126" s="35"/>
+      <c r="F126" s="34"/>
     </row>
     <row r="127" spans="1:6">
-      <c r="A127" s="35"/>
-      <c r="B127" s="58"/>
-      <c r="C127" s="61"/>
-      <c r="D127" s="35"/>
-      <c r="E127" s="35"/>
-      <c r="F127" s="35"/>
+      <c r="A127" s="34"/>
+      <c r="B127" s="38"/>
+      <c r="C127" s="41"/>
+      <c r="D127" s="34"/>
+      <c r="E127" s="34"/>
+      <c r="F127" s="34"/>
     </row>
     <row r="128" spans="1:6">
-      <c r="A128" s="35"/>
-      <c r="B128" s="58"/>
-      <c r="C128" s="61"/>
-      <c r="D128" s="35"/>
-      <c r="E128" s="35"/>
-      <c r="F128" s="35"/>
+      <c r="A128" s="34"/>
+      <c r="B128" s="38"/>
+      <c r="C128" s="41"/>
+      <c r="D128" s="34"/>
+      <c r="E128" s="34"/>
+      <c r="F128" s="34"/>
     </row>
     <row r="129" spans="1:8" ht="165">
-      <c r="A129" s="35"/>
-      <c r="B129" s="58"/>
-      <c r="C129" s="61"/>
-      <c r="D129" s="35"/>
-      <c r="E129" s="36" t="s">
+      <c r="A129" s="34"/>
+      <c r="B129" s="38"/>
+      <c r="C129" s="41"/>
+      <c r="D129" s="34"/>
+      <c r="E129" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="F129" s="37" t="s">
+      <c r="F129" s="36" t="s">
         <v>159</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="60">
-      <c r="A130" s="35"/>
-      <c r="B130" s="58"/>
-      <c r="C130" s="61"/>
-      <c r="D130" s="35"/>
-      <c r="E130" s="37" t="s">
+      <c r="A130" s="34"/>
+      <c r="B130" s="38"/>
+      <c r="C130" s="41"/>
+      <c r="D130" s="34"/>
+      <c r="E130" s="36" t="s">
         <v>160</v>
       </c>
-      <c r="F130" s="35"/>
+      <c r="F130" s="34"/>
     </row>
     <row r="131" spans="1:8">
-      <c r="A131" s="35"/>
-      <c r="B131" s="58"/>
-      <c r="C131" s="61"/>
-      <c r="D131" s="35" t="s">
+      <c r="A131" s="34"/>
+      <c r="B131" s="38"/>
+      <c r="C131" s="41"/>
+      <c r="D131" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="E131" s="35" t="s">
+      <c r="E131" s="34" t="s">
         <v>161</v>
       </c>
-      <c r="F131" s="35"/>
+      <c r="F131" s="34"/>
     </row>
     <row r="132" spans="1:8">
-      <c r="A132" s="35"/>
-      <c r="B132" s="58"/>
-      <c r="C132" s="61"/>
-      <c r="D132" s="35" t="s">
+      <c r="A132" s="34"/>
+      <c r="B132" s="38"/>
+      <c r="C132" s="41"/>
+      <c r="D132" s="34" t="s">
         <v>101</v>
       </c>
-      <c r="E132" s="35" t="s">
+      <c r="E132" s="34" t="s">
         <v>162</v>
       </c>
-      <c r="F132" s="35"/>
+      <c r="F132" s="34"/>
     </row>
     <row r="133" spans="1:8">
-      <c r="A133" s="35"/>
-      <c r="B133" s="58"/>
-      <c r="C133" s="61"/>
-      <c r="D133" s="35"/>
-      <c r="E133" s="35" t="s">
+      <c r="A133" s="34"/>
+      <c r="B133" s="38"/>
+      <c r="C133" s="41"/>
+      <c r="D133" s="34"/>
+      <c r="E133" s="34" t="s">
         <v>163</v>
       </c>
-      <c r="F133" s="35"/>
+      <c r="F133" s="34"/>
     </row>
     <row r="134" spans="1:8" ht="45">
-      <c r="A134" s="35"/>
-      <c r="B134" s="58"/>
-      <c r="C134" s="61"/>
-      <c r="D134" s="35" t="s">
+      <c r="A134" s="34"/>
+      <c r="B134" s="38"/>
+      <c r="C134" s="41"/>
+      <c r="D134" s="34" t="s">
         <v>130</v>
       </c>
-      <c r="E134" s="37" t="s">
+      <c r="E134" s="36" t="s">
         <v>164</v>
       </c>
-      <c r="F134" s="35"/>
+      <c r="F134" s="34"/>
     </row>
     <row r="135" spans="1:8">
-      <c r="A135" s="35"/>
-      <c r="B135" s="58"/>
-      <c r="C135" s="61"/>
-      <c r="D135" s="35"/>
-      <c r="E135" s="35"/>
-      <c r="F135" s="35"/>
+      <c r="A135" s="34"/>
+      <c r="B135" s="38"/>
+      <c r="C135" s="41"/>
+      <c r="D135" s="34"/>
+      <c r="E135" s="34"/>
+      <c r="F135" s="34"/>
     </row>
     <row r="136" spans="1:8" ht="45">
-      <c r="A136" s="35"/>
-      <c r="B136" s="58"/>
-      <c r="C136" s="61"/>
-      <c r="D136" s="35"/>
-      <c r="E136" s="37" t="s">
+      <c r="A136" s="34"/>
+      <c r="B136" s="38"/>
+      <c r="C136" s="41"/>
+      <c r="D136" s="34"/>
+      <c r="E136" s="36" t="s">
         <v>165</v>
       </c>
-      <c r="F136" s="37" t="s">
+      <c r="F136" s="36" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="45">
-      <c r="A137" s="35"/>
-      <c r="B137" s="59"/>
-      <c r="C137" s="62"/>
-      <c r="D137" s="35"/>
-      <c r="E137" s="36" t="s">
+      <c r="A137" s="34"/>
+      <c r="B137" s="39"/>
+      <c r="C137" s="42"/>
+      <c r="D137" s="34"/>
+      <c r="E137" s="35" t="s">
         <v>167</v>
       </c>
-      <c r="F137" s="37" t="s">
+      <c r="F137" s="36" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="75">
-      <c r="B138" s="31">
+      <c r="A138" s="31"/>
+      <c r="B138" s="50">
         <v>46295</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C138" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="E138" s="21" t="s">
+      <c r="D138" s="31"/>
+      <c r="E138" s="33" t="s">
         <v>169</v>
       </c>
-      <c r="F138" s="22" t="s">
+      <c r="F138" s="32" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="60">
-      <c r="E139" s="21" t="s">
+      <c r="A139" s="31"/>
+      <c r="B139" s="51"/>
+      <c r="C139" s="54"/>
+      <c r="D139" s="31"/>
+      <c r="E139" s="33" t="s">
         <v>171</v>
       </c>
-      <c r="F139" s="22" t="s">
+      <c r="F139" s="32" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="75">
-      <c r="E140" s="21" t="s">
+      <c r="A140" s="31"/>
+      <c r="B140" s="51"/>
+      <c r="C140" s="54"/>
+      <c r="D140" s="31"/>
+      <c r="E140" s="33" t="s">
         <v>172</v>
       </c>
-      <c r="F140" s="22" t="s">
+      <c r="F140" s="32" t="s">
         <v>173</v>
       </c>
     </row>
+    <row r="141" spans="1:8">
+      <c r="A141" s="31"/>
+      <c r="B141" s="51"/>
+      <c r="C141" s="54"/>
+      <c r="D141" s="31"/>
+      <c r="E141" s="31"/>
+      <c r="F141" s="31"/>
+    </row>
     <row r="142" spans="1:8" ht="60">
-      <c r="E142" s="21" t="s">
+      <c r="A142" s="31"/>
+      <c r="B142" s="51"/>
+      <c r="C142" s="54"/>
+      <c r="D142" s="31"/>
+      <c r="E142" s="33" t="s">
         <v>175</v>
       </c>
-      <c r="F142" s="38" t="s">
+      <c r="F142" s="61" t="s">
+        <v>179</v>
+      </c>
+      <c r="H142" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="H142" s="22" t="s">
+    </row>
+    <row r="143" spans="1:8" ht="75">
+      <c r="A143" s="31"/>
+      <c r="B143" s="51"/>
+      <c r="C143" s="54"/>
+      <c r="D143" s="31"/>
+      <c r="E143" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="F143" s="32" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="144" spans="1:8">
+      <c r="A144" s="31"/>
+      <c r="B144" s="51"/>
+      <c r="C144" s="54"/>
+      <c r="D144" s="31"/>
+      <c r="E144" s="31"/>
+      <c r="F144" s="31"/>
+    </row>
+    <row r="145" spans="1:8" ht="60">
+      <c r="A145" s="31"/>
+      <c r="B145" s="51"/>
+      <c r="C145" s="54"/>
+      <c r="D145" s="31"/>
+      <c r="E145" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="F145" s="61" t="s">
+        <v>178</v>
+      </c>
+      <c r="H145" s="21" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8">
+      <c r="A146" s="31"/>
+      <c r="B146" s="52"/>
+      <c r="C146" s="55"/>
+      <c r="D146" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="E146" s="31" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="143" spans="1:8" ht="90">
-      <c r="E143" s="22" t="s">
-        <v>176</v>
-      </c>
-      <c r="F143" s="22" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="145" spans="4:8" ht="60">
-      <c r="E145" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="F145" s="38" t="s">
-        <v>179</v>
-      </c>
-      <c r="H145" s="22" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="146" spans="4:8">
-      <c r="D146" t="s">
-        <v>102</v>
-      </c>
-      <c r="E146" t="s">
-        <v>182</v>
+      <c r="F146" s="31"/>
+    </row>
+    <row r="147" spans="1:8" ht="60">
+      <c r="B147" s="30">
+        <v>46266</v>
+      </c>
+      <c r="D147" t="s">
+        <v>185</v>
+      </c>
+      <c r="E147" s="21" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" ht="75">
+      <c r="E148" s="21" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8">
+      <c r="B150" s="30">
+        <v>46270</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8">
+      <c r="B151" s="30">
+        <v>46271</v>
+      </c>
+      <c r="D151" t="s">
+        <v>117</v>
+      </c>
+      <c r="E151" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" ht="45">
+      <c r="B152" s="30">
+        <v>46271</v>
+      </c>
+      <c r="E152" s="21" t="s">
+        <v>187</v>
+      </c>
+      <c r="F152" s="21" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" ht="45">
+      <c r="E153" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="F153" s="21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" ht="75">
+      <c r="E154" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="F154" s="21" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" ht="45">
+      <c r="E155" s="21" t="s">
+        <v>192</v>
+      </c>
+      <c r="F155" s="21" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="45">
+      <c r="D156" t="s">
+        <v>101</v>
+      </c>
+      <c r="E156" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="F156" s="21" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" ht="30">
+      <c r="E157" s="21" t="s">
+        <v>197</v>
+      </c>
+      <c r="F157" s="21" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:F90" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="50">
+  <mergeCells count="52">
+    <mergeCell ref="C138:C146"/>
+    <mergeCell ref="B138:B146"/>
+    <mergeCell ref="B110:B121"/>
+    <mergeCell ref="C110:C121"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="C90:C94"/>
+    <mergeCell ref="B90:B95"/>
+    <mergeCell ref="B78:B83"/>
+    <mergeCell ref="C78:C83"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="C84:C89"/>
+    <mergeCell ref="B96:B109"/>
+    <mergeCell ref="C96:C109"/>
+    <mergeCell ref="C39:C45"/>
+    <mergeCell ref="D39:D45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D71:D77"/>
+    <mergeCell ref="B52:B57"/>
+    <mergeCell ref="C52:C57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="C62:C66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="C67:C70"/>
+    <mergeCell ref="B71:B77"/>
+    <mergeCell ref="C71:C77"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="D3:D7"/>
+    <mergeCell ref="B8:B16"/>
+    <mergeCell ref="C8:C16"/>
     <mergeCell ref="B122:B137"/>
     <mergeCell ref="C122:C137"/>
     <mergeCell ref="D26:D29"/>
@@ -4460,40 +4768,6 @@
     <mergeCell ref="C34:C38"/>
     <mergeCell ref="D34:D38"/>
     <mergeCell ref="B39:B45"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="D3:D7"/>
-    <mergeCell ref="B8:B16"/>
-    <mergeCell ref="C8:C16"/>
-    <mergeCell ref="C39:C45"/>
-    <mergeCell ref="D39:D45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="D71:D77"/>
-    <mergeCell ref="B52:B57"/>
-    <mergeCell ref="C52:C57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="C62:C66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="C67:C70"/>
-    <mergeCell ref="B71:B77"/>
-    <mergeCell ref="C71:C77"/>
-    <mergeCell ref="B110:B121"/>
-    <mergeCell ref="C110:C121"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="C90:C94"/>
-    <mergeCell ref="B90:B95"/>
-    <mergeCell ref="B78:B83"/>
-    <mergeCell ref="C78:C83"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="C84:C89"/>
-    <mergeCell ref="B96:B109"/>
-    <mergeCell ref="C96:C109"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
Restore local changes and update seed files 23-10-2026 Laxmi
</commit_message>
<xml_diff>
--- a/Action_Items_Tracking_Sheet_Formatted.xlsx
+++ b/Action_Items_Tracking_Sheet_Formatted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AITO-Recovered\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE14822-E10F-4877-B962-0E74C7B86137}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC043AA0-B924-4567-A3DE-BB700198AECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="263">
   <si>
     <t>Action Items &amp; Work Hours Tracking Log</t>
   </si>
@@ -563,33 +563,6 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve"> Enable Single-Click Role Selection and Navigation to Choose Activities</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>..in workflow role 
-selctor page. (in app)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Task Name:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
       <t xml:space="preserve"> Update </t>
     </r>
     <r>
@@ -787,84 +760,10 @@
     </r>
   </si>
   <si>
-    <t>Currently, some applicable agents such as **Sales Home are not being identified or displayed under 
-Primary/Secondary Tools and the Resources tab**, and the task is to investigate why this is 
-happening across roles/topics and fix the underlying mapping/filtering issue.     (in-app)</t>
-  </si>
-  <si>
     <t>Remove logo in the html page</t>
   </si>
   <si>
     <t>5 mins</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Remove the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>“All Roles”</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> option from the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>Role Path</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> page while keeping it available on the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t>All Topics</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> page.
-(in-app &amp; main app)</t>
-    </r>
   </si>
   <si>
     <r>
@@ -1764,6 +1663,569 @@
   </si>
   <si>
     <t>verfiy in main app</t>
+  </si>
+  <si>
+    <t>Resolved Merge conflicts.</t>
+  </si>
+  <si>
+    <t>1hr 30</t>
+  </si>
+  <si>
+    <t>need to verify in in-app</t>
+  </si>
+  <si>
+    <t>in main app</t>
+  </si>
+  <si>
+    <t>in In app</t>
+  </si>
+  <si>
+    <r>
+      <t>Task Name:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Enable Single-Click Role Selection and Navigation to Choose Activities</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">..in workflow role 
+selctor page. (in app) </t>
+    </r>
+  </si>
+  <si>
+    <t>both in in-app
+ and main app</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Fix the issue where a topic selected under one </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Audience</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> remains highlighted after clearing or changing the Audience filter, causing incorrect topic selection across different audiences.</t>
+    </r>
+  </si>
+  <si>
+    <t>Fix the issue where a topic selected under Manager remains selected in All Topics after switching
+ to the Facilitator role.  (All Topics Page) (drop down and topic issue)</t>
+  </si>
+  <si>
+    <t>In App</t>
+  </si>
+  <si>
+    <t>Task Name: Fix Side Panel Behavior When Deselecting Topics on the "All Topics" Page.currently if 
+ you select one topic and deselct it it is showing the side panel. Fix that in case of selecting multiple topics</t>
+  </si>
+  <si>
+    <t>already implemented in in-app now implemented in main app</t>
+  </si>
+  <si>
+    <t>Currently, some applicable agents such as  "Sales Home are not being identified or displayed under 
+Primary/Secondary Tools and the Resources tab", and the task is to investigate why this is 
+happening across roles/topics and fix the underlying mapping/filtering issue.     (in-app)</t>
+  </si>
+  <si>
+    <t>need to 
+implement in main app</t>
+  </si>
+  <si>
+    <t>Remove the “All Roles” option from the Role Path page while keeping it available on the All Topics page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implemented pending item in main app </t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Remove the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>“All Roles”</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> option from the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>Role Path</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> page while keeping it available on the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>All Topics</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> page.
+(in-app).</t>
+    </r>
+  </si>
+  <si>
+    <t>start from here</t>
+  </si>
+  <si>
+    <t>All Hands meeting</t>
+  </si>
+  <si>
+    <t>Wed</t>
+  </si>
+  <si>
+    <t>Investigated the entire pipeline code developed by tech team</t>
+  </si>
+  <si>
+    <t>Audited and enhanced the existing Tips/Walkthrough feature to identify and implement missing, outdated, and broken tips across pages, buttons, cards, and workflows, ensuring accurate guidance for new users and role-specific features.</t>
+  </si>
+  <si>
+    <t>meet with nihar regarding Sandbox database</t>
+  </si>
+  <si>
+    <t>2 hr 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Investigated CD pipeline code </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1hr </t>
+  </si>
+  <si>
+    <t>SQL learnings on QUERY &amp; OPTIMIZATION</t>
+  </si>
+  <si>
+    <t>SQL learnings on QUERY &amp; OPTIMIZATION (Practical Implementation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">implemented main app changes </t>
+  </si>
+  <si>
+    <t>Extended the existing guided walkthrough to include Step 6 – Profile Settings &amp; Feedback, highlighting the profile menu and Send feedback option while preserving all existing features and functionality.</t>
+  </si>
+  <si>
+    <t>learnings</t>
+  </si>
+  <si>
+    <t>2-4:50</t>
+  </si>
+  <si>
+    <t>5:30-6:30</t>
+  </si>
+  <si>
+    <t>meet with nihar regarding Sandbox database,ran cd pipelines for qa environment</t>
+  </si>
+  <si>
+    <t>answering questions of privacy review</t>
+  </si>
+  <si>
+    <t>created a data flow diagram for our application</t>
+  </si>
+  <si>
+    <t>meet with brahmam</t>
+  </si>
+  <si>
+    <t>1 hr 30</t>
+  </si>
+  <si>
+    <t>Validated client's generated data flow diagram.</t>
+  </si>
+  <si>
+    <t>The current walkthrough displays the “Create your own huddle” tip as the second step, while essential navigation and page-orientation guidance need higher priority. Reordered the tips to show essential guidance first and moved the huddle creation tip to the final step, removing unnecessary tips without affecting other features.</t>
+  </si>
+  <si>
+    <t>need to
+ implement in main app</t>
+  </si>
+  <si>
+    <t>prompt in team's chat</t>
+  </si>
+  <si>
+    <t>Updated the Facilitator Hub to display Primary AI Tools and Secondary AI Tools in separate sections
+ instead of combining them under Key AI Tools. Ensured tools are categorized using existing application
+ data while preserving other features and UI functionality.</t>
+  </si>
+  <si>
+    <t>Compared the existing application data with the newly provided Excel workbook to identify missing, 
+outdated, mismatched, and additional records. Updated the application data file and made 
+the necessary UI and data-mapping changes to align the application with the new workbook 
+while preserving existing functionality.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Huddle segment and role updates are also appearing in Workflow Builder, which should retain only its original Enterprise and Manager segments.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Expected behavior:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Keep Workflow and Huddle role lists separate so changes in one module do not affect the other, without breaking existing functionality.</t>
+    </r>
+  </si>
+  <si>
+    <t>need to implement in main app</t>
+  </si>
+  <si>
+    <t>**Task: Update Five Incorrect Huddle Role Path Placements Using the Latest Excel Workbook**
+**Current Scenario:**
+The AITO Huddle Generator application is displaying older or incorrect placement content for five role/week combinations. The latest workbook, `Frontier_Accelerator_Huddle_App_Content_Integration_Model_10.13.2026 v2.xlsx`, contains the updated placements, but these placement IDs and their corresponding content are missing from the application's runtime data and role/week mappings.
+The affected placements are `DAE-W06`, `CE-W02`, `CE-W07`, `DSE-W06`, and `DCSA-W02`. Although the corresponding weeks are visible in the application, they display older placements or different titles instead of the latest workbook content.
+**Required Fix:**
+Update the application's runtime data and relevant role/week mappings using the exact content from the workbook's `Role_Paths` sheet. Ensure that each placement is associated with the correct role and week and that the UI displays the updated title, description, objective, WIIFM text, and other required fields.
+Validate the changes against the workbook and verify that all five placements display correctly in the application. Preserve existing functionality, keep Workflow Builder and Huddle Generator roles separate, and avoid modifying unrelated data, features, or files.</t>
+  </si>
+  <si>
+    <t>Currently, 19 resources in the Excel workbook are not linked to any topic or activity, so they are not easily accessible through the Huddle page. Update the existing Resources button to display these resources globally for all roles, without changing any other features.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Task Name: Fully Synchronize AITO Huddle Generator Data with the Latest Excel Workbook:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">
+Synchronize AITO Huddle Generator data with the latest Excel workbook, updating outdated topics, activities, placements, DSS content, and role/week mappings while removing obsolete records.
+Validate all changes against the workbook and run available tests and builds. Keep changes limited to Huddle data and required runtime logic, preserve unrelated functionality, and do not commit or push changes.</t>
+    </r>
+  </si>
+  <si>
+    <t>Issue</t>
+  </si>
+  <si>
+    <t>Existing Mapping Logic</t>
+  </si>
+  <si>
+    <r>
+      <t>Role_Paths:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Identifies the role, week, and associated topic/placement.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Activities:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Provides the activities associated with the selected placement.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Activity_Agents:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Maps each Activity ID to its assigned Agent ID and usage type (Primary or Secondary).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Topic_Agents:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Stores topic-level tool mappings, which may include tools not assigned to the selected huddle's activities.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Agents:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Maps Agent IDs to readable tool names.</t>
+    </r>
+  </si>
+  <si>
+    <t>Implementation</t>
+  </si>
+  <si>
+    <t>Remaining Work</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Task Name:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Fix Huddle Tool Mapping Logic to Use Activity-Level Assignments</t>
+    </r>
+  </si>
+  <si>
+    <t>Currently, the application uses a combination of activity-level and topic-level mappings to display 
+AI tools for a specific role-path week. Primary tools are fetched from activity-level mappings, while
+ Secondary tools are fetched from topic-level mappings. This can cause tools that are associated with
+ a topic generally, but are not assigned to that specific huddle's activities, to appear in the UI.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Previously, the application fetched Primary tools from </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Activity_Agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> but fetched Secondary tools from
+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Topic_Agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>. As a result, unrelated topic-level tools could appear as Secondary tools for a specific role-path week.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The tool-mapping logic has been updated in the Standalone application to use </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Activity_Agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> as
+ the source for both Primary and Secondary tools. The application identifies the activities belonging
+ to the selected placement and retrieves their assigned tools and usage types from the activity-level mappings.</t>
+    </r>
+  </si>
+  <si>
+    <t>This ensures that both Primary and Secondary tools are based on the activities assigned to that specific
+ role-path week, rather than including tools simply because they are associated with the broader topic.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Apply the same mapping-logic change to the main application (.NET backend and SQL Server). 
+Update the backend logic so that both Primary and Secondary tools are derived from
+ activity-level assignments in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Activity_Agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>/the corresponding activity-agent database mappings,
+ instead of deriving Secondary tools from topic-level mappings.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Both the Standalone and main applications should display tools consistently and only use activity-level
+ assignments for the selected role-path placement. Topic-level mappings in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>Topic_Agents</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> should not
+ independently introduce tools into the huddle's Primary or Secondary lists.</t>
+    </r>
+  </si>
+  <si>
+    <t>Worked on UAT DEPLOYMENT PROCESS.</t>
   </si>
 </sst>
 </file>
@@ -1774,7 +2236,7 @@
     <numFmt numFmtId="164" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0&quot; h&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1854,8 +2316,29 @@
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1931,6 +2414,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2027,7 +2516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2123,6 +2612,85 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="14" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="14" fontId="0" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2132,6 +2700,30 @@
     <xf numFmtId="14" fontId="0" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2141,62 +2733,8 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2465,7 +3003,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H157"/>
+  <dimension ref="A1:I229"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -2474,18 +3012,18 @@
     <col min="4" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="95" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="3.85546875" customWidth="1"/>
+    <col min="7" max="7" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="69" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-      <c r="F1" s="49"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
     </row>
     <row r="2" spans="1:6" ht="21.75" customHeight="1">
       <c r="A2" s="3" t="s">
@@ -2511,13 +3049,13 @@
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="44">
+      <c r="B3" s="53">
         <v>46260</v>
       </c>
-      <c r="C3" s="46" t="s">
+      <c r="C3" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="43">
+      <c r="D3" s="70">
         <v>6.5</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -2531,9 +3069,9 @@
       <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
       <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
@@ -2545,9 +3083,9 @@
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="44"/>
-      <c r="C5" s="44"/>
-      <c r="D5" s="44"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
       <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
@@ -2559,9 +3097,9 @@
       <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="44"/>
-      <c r="C6" s="44"/>
-      <c r="D6" s="44"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
       <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
@@ -2573,9 +3111,9 @@
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="44"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
       <c r="E7" s="4" t="s">
         <v>13</v>
       </c>
@@ -2587,10 +3125,10 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="45">
+      <c r="B8" s="51">
         <v>46261</v>
       </c>
-      <c r="C8" s="47" t="s">
+      <c r="C8" s="52" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -2607,8 +3145,8 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="45"/>
-      <c r="C9" s="45"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="51"/>
       <c r="D9" s="1" t="s">
         <v>111</v>
       </c>
@@ -2623,8 +3161,8 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="45"/>
-      <c r="C10" s="45"/>
+      <c r="B10" s="51"/>
+      <c r="C10" s="51"/>
       <c r="D10" s="1" t="s">
         <v>99</v>
       </c>
@@ -2639,8 +3177,8 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="45"/>
-      <c r="C11" s="45"/>
+      <c r="B11" s="51"/>
+      <c r="C11" s="51"/>
       <c r="D11" s="1" t="s">
         <v>101</v>
       </c>
@@ -2655,8 +3193,8 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="45"/>
-      <c r="C12" s="45"/>
+      <c r="B12" s="51"/>
+      <c r="C12" s="51"/>
       <c r="D12" s="1" t="s">
         <v>109</v>
       </c>
@@ -2671,8 +3209,8 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="45"/>
-      <c r="C13" s="45"/>
+      <c r="B13" s="51"/>
+      <c r="C13" s="51"/>
       <c r="D13" s="1" t="s">
         <v>109</v>
       </c>
@@ -2687,8 +3225,8 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45"/>
+      <c r="B14" s="51"/>
+      <c r="C14" s="51"/>
       <c r="D14" s="1" t="s">
         <v>99</v>
       </c>
@@ -2703,8 +3241,8 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="45"/>
-      <c r="C15" s="45"/>
+      <c r="B15" s="51"/>
+      <c r="C15" s="51"/>
       <c r="D15" s="1" t="s">
         <v>101</v>
       </c>
@@ -2719,8 +3257,8 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="45"/>
-      <c r="C16" s="45"/>
+      <c r="B16" s="51"/>
+      <c r="C16" s="51"/>
       <c r="D16" s="1" t="s">
         <v>101</v>
       </c>
@@ -2735,10 +3273,10 @@
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="44">
+      <c r="B17" s="53">
         <v>46266</v>
       </c>
-      <c r="C17" s="46" t="s">
+      <c r="C17" s="54" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -2755,8 +3293,8 @@
       <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="44"/>
-      <c r="C18" s="44"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
       <c r="D18" s="2" t="s">
         <v>103</v>
       </c>
@@ -2771,8 +3309,8 @@
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="44"/>
-      <c r="C19" s="44"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="53"/>
       <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
@@ -2787,8 +3325,8 @@
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="44"/>
-      <c r="C20" s="44"/>
+      <c r="B20" s="53"/>
+      <c r="C20" s="53"/>
       <c r="D20" s="2" t="s">
         <v>112</v>
       </c>
@@ -2803,10 +3341,10 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="45">
+      <c r="B21" s="51">
         <v>46267</v>
       </c>
-      <c r="C21" s="47" t="s">
+      <c r="C21" s="52" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -2823,8 +3361,8 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="45"/>
-      <c r="C22" s="45"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="51"/>
       <c r="D22" s="1" t="s">
         <v>102</v>
       </c>
@@ -2839,8 +3377,8 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="45"/>
-      <c r="C23" s="45"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="51"/>
       <c r="D23" s="1" t="s">
         <v>101</v>
       </c>
@@ -2855,8 +3393,8 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="45"/>
-      <c r="C24" s="45"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
       <c r="D24" s="1" t="s">
         <v>101</v>
       </c>
@@ -2871,8 +3409,8 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="45"/>
-      <c r="C25" s="45"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
       <c r="D25" s="1" t="s">
         <v>101</v>
       </c>
@@ -2887,13 +3425,13 @@
       <c r="A26" s="2">
         <v>24</v>
       </c>
-      <c r="B26" s="44">
+      <c r="B26" s="53">
         <v>46268</v>
       </c>
-      <c r="C26" s="46" t="s">
+      <c r="C26" s="54" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="43">
+      <c r="D26" s="70">
         <v>7</v>
       </c>
       <c r="E26" s="4" t="s">
@@ -2907,9 +3445,9 @@
       <c r="A27" s="2">
         <v>25</v>
       </c>
-      <c r="B27" s="44"/>
-      <c r="C27" s="44"/>
-      <c r="D27" s="44"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
       <c r="E27" s="4" t="s">
         <v>36</v>
       </c>
@@ -2921,9 +3459,9 @@
       <c r="A28" s="2">
         <v>26</v>
       </c>
-      <c r="B28" s="44"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="44"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="53"/>
       <c r="E28" s="4" t="s">
         <v>37</v>
       </c>
@@ -2935,9 +3473,9 @@
       <c r="A29" s="2">
         <v>27</v>
       </c>
-      <c r="B29" s="44"/>
-      <c r="C29" s="44"/>
-      <c r="D29" s="44"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="53"/>
+      <c r="D29" s="53"/>
       <c r="E29" s="4" t="s">
         <v>38</v>
       </c>
@@ -2949,13 +3487,13 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="45">
+      <c r="B30" s="51">
         <v>46269</v>
       </c>
-      <c r="C30" s="47" t="s">
+      <c r="C30" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="48">
+      <c r="D30" s="80">
         <v>7</v>
       </c>
       <c r="E30" s="6" t="s">
@@ -2969,9 +3507,9 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="45"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
       <c r="E31" s="6" t="s">
         <v>41</v>
       </c>
@@ -2983,9 +3521,9 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="45"/>
-      <c r="C32" s="45"/>
-      <c r="D32" s="45"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="51"/>
       <c r="E32" s="6" t="s">
         <v>42</v>
       </c>
@@ -2997,9 +3535,9 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="45"/>
-      <c r="C33" s="45"/>
-      <c r="D33" s="45"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="51"/>
       <c r="E33" s="6" t="s">
         <v>43</v>
       </c>
@@ -3011,13 +3549,13 @@
       <c r="A34" s="2">
         <v>32</v>
       </c>
-      <c r="B34" s="44">
+      <c r="B34" s="53">
         <v>46272</v>
       </c>
-      <c r="C34" s="46" t="s">
+      <c r="C34" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="43">
+      <c r="D34" s="70">
         <v>8</v>
       </c>
       <c r="E34" s="4" t="s">
@@ -3031,9 +3569,9 @@
       <c r="A35" s="2">
         <v>33</v>
       </c>
-      <c r="B35" s="44"/>
-      <c r="C35" s="44"/>
-      <c r="D35" s="44"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
       <c r="E35" s="4" t="s">
         <v>46</v>
       </c>
@@ -3045,9 +3583,9 @@
       <c r="A36" s="2">
         <v>34</v>
       </c>
-      <c r="B36" s="44"/>
-      <c r="C36" s="44"/>
-      <c r="D36" s="44"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
       <c r="E36" s="4" t="s">
         <v>47</v>
       </c>
@@ -3059,9 +3597,9 @@
       <c r="A37" s="2">
         <v>35</v>
       </c>
-      <c r="B37" s="44"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="44"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
       <c r="E37" s="4" t="s">
         <v>48</v>
       </c>
@@ -3073,9 +3611,9 @@
       <c r="A38" s="2">
         <v>36</v>
       </c>
-      <c r="B38" s="44"/>
-      <c r="C38" s="44"/>
-      <c r="D38" s="44"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
       <c r="E38" s="4" t="s">
         <v>49</v>
       </c>
@@ -3087,13 +3625,13 @@
       <c r="A39" s="1">
         <v>37</v>
       </c>
-      <c r="B39" s="45">
+      <c r="B39" s="51">
         <v>46273</v>
       </c>
-      <c r="C39" s="47" t="s">
+      <c r="C39" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="D39" s="48">
+      <c r="D39" s="80">
         <v>6</v>
       </c>
       <c r="E39" s="6" t="s">
@@ -3107,9 +3645,9 @@
       <c r="A40" s="1">
         <v>38</v>
       </c>
-      <c r="B40" s="45"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="45"/>
+      <c r="B40" s="51"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="51"/>
       <c r="E40" s="6" t="s">
         <v>51</v>
       </c>
@@ -3121,9 +3659,9 @@
       <c r="A41" s="1">
         <v>39</v>
       </c>
-      <c r="B41" s="45"/>
-      <c r="C41" s="45"/>
-      <c r="D41" s="45"/>
+      <c r="B41" s="51"/>
+      <c r="C41" s="51"/>
+      <c r="D41" s="51"/>
       <c r="E41" s="6" t="s">
         <v>52</v>
       </c>
@@ -3135,9 +3673,9 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" s="45"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="45"/>
+      <c r="B42" s="51"/>
+      <c r="C42" s="51"/>
+      <c r="D42" s="51"/>
       <c r="E42" s="6" t="s">
         <v>53</v>
       </c>
@@ -3149,9 +3687,9 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" s="45"/>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
+      <c r="B43" s="51"/>
+      <c r="C43" s="51"/>
+      <c r="D43" s="51"/>
       <c r="E43" s="6" t="s">
         <v>54</v>
       </c>
@@ -3163,9 +3701,9 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" s="45"/>
-      <c r="C44" s="45"/>
-      <c r="D44" s="45"/>
+      <c r="B44" s="51"/>
+      <c r="C44" s="51"/>
+      <c r="D44" s="51"/>
       <c r="E44" s="6" t="s">
         <v>55</v>
       </c>
@@ -3177,9 +3715,9 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" s="45"/>
-      <c r="C45" s="45"/>
-      <c r="D45" s="45"/>
+      <c r="B45" s="51"/>
+      <c r="C45" s="51"/>
+      <c r="D45" s="51"/>
       <c r="E45" s="6" t="s">
         <v>56</v>
       </c>
@@ -3191,10 +3729,10 @@
       <c r="A46" s="2">
         <v>44</v>
       </c>
-      <c r="B46" s="44">
+      <c r="B46" s="53">
         <v>46274</v>
       </c>
-      <c r="C46" s="46" t="s">
+      <c r="C46" s="54" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="2" t="s">
@@ -3211,8 +3749,8 @@
       <c r="A47" s="2">
         <v>45</v>
       </c>
-      <c r="B47" s="44"/>
-      <c r="C47" s="44"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="53"/>
       <c r="D47" s="2" t="s">
         <v>99</v>
       </c>
@@ -3225,8 +3763,8 @@
     </row>
     <row r="48" spans="1:6" ht="34.5" customHeight="1">
       <c r="A48" s="2"/>
-      <c r="B48" s="44"/>
-      <c r="C48" s="44"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="53"/>
       <c r="D48" s="2" t="s">
         <v>102</v>
       </c>
@@ -3239,8 +3777,8 @@
       <c r="A49" s="2">
         <v>46</v>
       </c>
-      <c r="B49" s="44"/>
-      <c r="C49" s="44"/>
+      <c r="B49" s="53"/>
+      <c r="C49" s="53"/>
       <c r="D49" s="2" t="s">
         <v>100</v>
       </c>
@@ -3252,13 +3790,13 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A50" s="47">
+      <c r="A50" s="52">
         <v>47</v>
       </c>
-      <c r="B50" s="45">
+      <c r="B50" s="51">
         <v>46275</v>
       </c>
-      <c r="C50" s="47" t="s">
+      <c r="C50" s="52" t="s">
         <v>14</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -3272,9 +3810,9 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A51" s="47"/>
-      <c r="B51" s="47"/>
-      <c r="C51" s="47"/>
+      <c r="A51" s="52"/>
+      <c r="B51" s="52"/>
+      <c r="C51" s="52"/>
       <c r="D51" s="1" t="s">
         <v>100</v>
       </c>
@@ -3289,10 +3827,10 @@
       <c r="A52" s="2">
         <v>49</v>
       </c>
-      <c r="B52" s="44">
+      <c r="B52" s="53">
         <v>46276</v>
       </c>
-      <c r="C52" s="46" t="s">
+      <c r="C52" s="54" t="s">
         <v>39</v>
       </c>
       <c r="D52" s="2" t="s">
@@ -3309,8 +3847,8 @@
       <c r="A53" s="2">
         <v>50</v>
       </c>
-      <c r="B53" s="44"/>
-      <c r="C53" s="44"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
       <c r="D53" s="2" t="s">
         <v>105</v>
       </c>
@@ -3325,8 +3863,8 @@
       <c r="A54" s="2">
         <v>51</v>
       </c>
-      <c r="B54" s="44"/>
-      <c r="C54" s="44"/>
+      <c r="B54" s="53"/>
+      <c r="C54" s="53"/>
       <c r="D54" s="2" t="s">
         <v>107</v>
       </c>
@@ -3341,8 +3879,8 @@
       <c r="A55" s="2">
         <v>52</v>
       </c>
-      <c r="B55" s="44"/>
-      <c r="C55" s="44"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="53"/>
       <c r="D55" s="2" t="s">
         <v>99</v>
       </c>
@@ -3355,8 +3893,8 @@
     </row>
     <row r="56" spans="1:6" ht="34.5" customHeight="1">
       <c r="A56" s="2"/>
-      <c r="B56" s="44"/>
-      <c r="C56" s="44"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="53"/>
       <c r="D56" s="2" t="s">
         <v>102</v>
       </c>
@@ -3369,8 +3907,8 @@
       <c r="A57" s="2">
         <v>53</v>
       </c>
-      <c r="B57" s="44"/>
-      <c r="C57" s="44"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="53"/>
       <c r="D57" s="2" t="s">
         <v>105</v>
       </c>
@@ -3385,10 +3923,10 @@
       <c r="A58" s="1">
         <v>54</v>
       </c>
-      <c r="B58" s="45">
+      <c r="B58" s="51">
         <v>46280</v>
       </c>
-      <c r="C58" s="47" t="s">
+      <c r="C58" s="52" t="s">
         <v>24</v>
       </c>
       <c r="D58" s="1" t="s">
@@ -3405,8 +3943,8 @@
       <c r="A59" s="1">
         <v>55</v>
       </c>
-      <c r="B59" s="45"/>
-      <c r="C59" s="45"/>
+      <c r="B59" s="51"/>
+      <c r="C59" s="51"/>
       <c r="D59" s="1" t="s">
         <v>102</v>
       </c>
@@ -3421,8 +3959,8 @@
       <c r="A60" s="1">
         <v>56</v>
       </c>
-      <c r="B60" s="45"/>
-      <c r="C60" s="45"/>
+      <c r="B60" s="51"/>
+      <c r="C60" s="51"/>
       <c r="D60" s="1" t="s">
         <v>105</v>
       </c>
@@ -3437,8 +3975,8 @@
       <c r="A61" s="1">
         <v>57</v>
       </c>
-      <c r="B61" s="45"/>
-      <c r="C61" s="45"/>
+      <c r="B61" s="51"/>
+      <c r="C61" s="51"/>
       <c r="D61" s="1" t="s">
         <v>106</v>
       </c>
@@ -3453,10 +3991,10 @@
       <c r="A62" s="2">
         <v>58</v>
       </c>
-      <c r="B62" s="44">
+      <c r="B62" s="53">
         <v>46281</v>
       </c>
-      <c r="C62" s="46" t="s">
+      <c r="C62" s="54" t="s">
         <v>7</v>
       </c>
       <c r="D62" s="2" t="s">
@@ -3473,8 +4011,8 @@
       <c r="A63" s="2">
         <v>59</v>
       </c>
-      <c r="B63" s="44"/>
-      <c r="C63" s="44"/>
+      <c r="B63" s="53"/>
+      <c r="C63" s="53"/>
       <c r="D63" s="2" t="s">
         <v>102</v>
       </c>
@@ -3489,8 +4027,8 @@
       <c r="A64" s="2">
         <v>60</v>
       </c>
-      <c r="B64" s="44"/>
-      <c r="C64" s="44"/>
+      <c r="B64" s="53"/>
+      <c r="C64" s="53"/>
       <c r="D64" s="2" t="s">
         <v>101</v>
       </c>
@@ -3505,8 +4043,8 @@
       <c r="A65" s="2">
         <v>61</v>
       </c>
-      <c r="B65" s="44"/>
-      <c r="C65" s="44"/>
+      <c r="B65" s="53"/>
+      <c r="C65" s="53"/>
       <c r="D65" s="2" t="s">
         <v>101</v>
       </c>
@@ -3521,8 +4059,8 @@
       <c r="A66" s="2">
         <v>62</v>
       </c>
-      <c r="B66" s="44"/>
-      <c r="C66" s="44"/>
+      <c r="B66" s="53"/>
+      <c r="C66" s="53"/>
       <c r="D66" s="2" t="s">
         <v>102</v>
       </c>
@@ -3537,10 +4075,10 @@
       <c r="A67" s="1">
         <v>63</v>
       </c>
-      <c r="B67" s="45">
+      <c r="B67" s="51">
         <v>46282</v>
       </c>
-      <c r="C67" s="47" t="s">
+      <c r="C67" s="52" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -3557,8 +4095,8 @@
       <c r="A68" s="1">
         <v>64</v>
       </c>
-      <c r="B68" s="45"/>
-      <c r="C68" s="45"/>
+      <c r="B68" s="51"/>
+      <c r="C68" s="51"/>
       <c r="D68" s="1" t="s">
         <v>105</v>
       </c>
@@ -3573,8 +4111,8 @@
       <c r="A69" s="1">
         <v>65</v>
       </c>
-      <c r="B69" s="45"/>
-      <c r="C69" s="45"/>
+      <c r="B69" s="51"/>
+      <c r="C69" s="51"/>
       <c r="D69" s="1" t="s">
         <v>102</v>
       </c>
@@ -3589,8 +4127,8 @@
       <c r="A70" s="1">
         <v>66</v>
       </c>
-      <c r="B70" s="45"/>
-      <c r="C70" s="45"/>
+      <c r="B70" s="51"/>
+      <c r="C70" s="51"/>
       <c r="D70" s="1" t="s">
         <v>104</v>
       </c>
@@ -3605,13 +4143,13 @@
       <c r="A71" s="2">
         <v>67</v>
       </c>
-      <c r="B71" s="44">
+      <c r="B71" s="53">
         <v>46283</v>
       </c>
-      <c r="C71" s="46" t="s">
+      <c r="C71" s="54" t="s">
         <v>39</v>
       </c>
-      <c r="D71" s="43">
+      <c r="D71" s="70">
         <v>7</v>
       </c>
       <c r="E71" s="4" t="s">
@@ -3625,9 +4163,9 @@
       <c r="A72" s="2">
         <v>68</v>
       </c>
-      <c r="B72" s="44"/>
-      <c r="C72" s="44"/>
-      <c r="D72" s="44"/>
+      <c r="B72" s="53"/>
+      <c r="C72" s="53"/>
+      <c r="D72" s="53"/>
       <c r="E72" s="4" t="s">
         <v>82</v>
       </c>
@@ -3639,9 +4177,9 @@
       <c r="A73" s="2">
         <v>69</v>
       </c>
-      <c r="B73" s="44"/>
-      <c r="C73" s="44"/>
-      <c r="D73" s="44"/>
+      <c r="B73" s="53"/>
+      <c r="C73" s="53"/>
+      <c r="D73" s="53"/>
       <c r="E73" s="4" t="s">
         <v>83</v>
       </c>
@@ -3653,9 +4191,9 @@
       <c r="A74" s="2">
         <v>70</v>
       </c>
-      <c r="B74" s="44"/>
-      <c r="C74" s="44"/>
-      <c r="D74" s="44"/>
+      <c r="B74" s="53"/>
+      <c r="C74" s="53"/>
+      <c r="D74" s="53"/>
       <c r="E74" s="4" t="s">
         <v>84</v>
       </c>
@@ -3667,9 +4205,9 @@
       <c r="A75" s="2">
         <v>71</v>
       </c>
-      <c r="B75" s="44"/>
-      <c r="C75" s="44"/>
-      <c r="D75" s="44"/>
+      <c r="B75" s="53"/>
+      <c r="C75" s="53"/>
+      <c r="D75" s="53"/>
       <c r="E75" s="4" t="s">
         <v>85</v>
       </c>
@@ -3681,9 +4219,9 @@
       <c r="A76" s="2">
         <v>72</v>
       </c>
-      <c r="B76" s="44"/>
-      <c r="C76" s="44"/>
-      <c r="D76" s="44"/>
+      <c r="B76" s="53"/>
+      <c r="C76" s="53"/>
+      <c r="D76" s="53"/>
       <c r="E76" s="4" t="s">
         <v>86</v>
       </c>
@@ -3695,9 +4233,9 @@
       <c r="A77" s="2">
         <v>73</v>
       </c>
-      <c r="B77" s="44"/>
-      <c r="C77" s="44"/>
-      <c r="D77" s="44"/>
+      <c r="B77" s="53"/>
+      <c r="C77" s="53"/>
+      <c r="D77" s="53"/>
       <c r="E77" s="4" t="s">
         <v>87</v>
       </c>
@@ -3709,10 +4247,10 @@
       <c r="A78" s="1">
         <v>74</v>
       </c>
-      <c r="B78" s="45">
+      <c r="B78" s="51">
         <v>46286</v>
       </c>
-      <c r="C78" s="47" t="s">
+      <c r="C78" s="52" t="s">
         <v>44</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -3729,8 +4267,8 @@
       <c r="A79" s="1">
         <v>75</v>
       </c>
-      <c r="B79" s="45"/>
-      <c r="C79" s="45"/>
+      <c r="B79" s="51"/>
+      <c r="C79" s="51"/>
       <c r="D79" s="1" t="s">
         <v>102</v>
       </c>
@@ -3745,8 +4283,8 @@
       <c r="A80" s="1">
         <v>76</v>
       </c>
-      <c r="B80" s="45"/>
-      <c r="C80" s="45"/>
+      <c r="B80" s="51"/>
+      <c r="C80" s="51"/>
       <c r="D80" s="1" t="s">
         <v>103</v>
       </c>
@@ -3757,12 +4295,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="78" customHeight="1">
+    <row r="81" spans="1:7" ht="78" customHeight="1">
       <c r="A81" s="1">
         <v>77</v>
       </c>
-      <c r="B81" s="45"/>
-      <c r="C81" s="45"/>
+      <c r="B81" s="51"/>
+      <c r="C81" s="51"/>
       <c r="D81" s="1" t="s">
         <v>102</v>
       </c>
@@ -3773,12 +4311,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="63.75" customHeight="1">
+    <row r="82" spans="1:7" ht="63.75" customHeight="1">
       <c r="A82" s="1">
         <v>78</v>
       </c>
-      <c r="B82" s="45"/>
-      <c r="C82" s="45"/>
+      <c r="B82" s="51"/>
+      <c r="C82" s="51"/>
       <c r="D82" s="1" t="s">
         <v>101</v>
       </c>
@@ -3789,12 +4327,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="34.5" customHeight="1">
+    <row r="83" spans="1:7" ht="34.5" customHeight="1">
       <c r="A83" s="1">
         <v>79</v>
       </c>
-      <c r="B83" s="45"/>
-      <c r="C83" s="45"/>
+      <c r="B83" s="51"/>
+      <c r="C83" s="51"/>
       <c r="D83" s="1" t="s">
         <v>102</v>
       </c>
@@ -3805,14 +4343,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="34.5" customHeight="1">
+    <row r="84" spans="1:7" ht="34.5" customHeight="1">
       <c r="A84" s="2">
         <v>80</v>
       </c>
-      <c r="B84" s="44">
+      <c r="B84" s="53">
         <v>46287</v>
       </c>
-      <c r="C84" s="46" t="s">
+      <c r="C84" s="54" t="s">
         <v>24</v>
       </c>
       <c r="D84" s="2" t="s">
@@ -3825,12 +4363,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="34.5" customHeight="1">
+    <row r="85" spans="1:7" ht="34.5" customHeight="1">
       <c r="A85" s="2">
         <v>81</v>
       </c>
-      <c r="B85" s="44"/>
-      <c r="C85" s="44"/>
+      <c r="B85" s="53"/>
+      <c r="C85" s="53"/>
       <c r="D85" s="2" t="s">
         <v>99</v>
       </c>
@@ -3841,12 +4379,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="194.25" customHeight="1">
+    <row r="86" spans="1:7" ht="194.25" customHeight="1">
       <c r="A86" s="2">
         <v>82</v>
       </c>
-      <c r="B86" s="44"/>
-      <c r="C86" s="44"/>
+      <c r="B86" s="53"/>
+      <c r="C86" s="53"/>
       <c r="D86" s="2" t="s">
         <v>100</v>
       </c>
@@ -3857,12 +4395,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="20.25" customHeight="1">
+    <row r="87" spans="1:7" ht="20.25" customHeight="1">
       <c r="A87" s="2">
         <v>83</v>
       </c>
-      <c r="B87" s="44"/>
-      <c r="C87" s="44"/>
+      <c r="B87" s="53"/>
+      <c r="C87" s="53"/>
       <c r="D87" s="2" t="s">
         <v>101</v>
       </c>
@@ -3873,10 +4411,10 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="20.25" customHeight="1">
+    <row r="88" spans="1:7" ht="20.25" customHeight="1">
       <c r="A88" s="2"/>
-      <c r="B88" s="44"/>
-      <c r="C88" s="44"/>
+      <c r="B88" s="53"/>
+      <c r="C88" s="53"/>
       <c r="D88" s="2" t="s">
         <v>101</v>
       </c>
@@ -3885,12 +4423,12 @@
       </c>
       <c r="F88" s="5"/>
     </row>
-    <row r="89" spans="1:6" ht="18.75" customHeight="1">
+    <row r="89" spans="1:7" ht="18.75" customHeight="1">
       <c r="A89" s="9">
         <v>84</v>
       </c>
-      <c r="B89" s="58"/>
-      <c r="C89" s="58"/>
+      <c r="B89" s="57"/>
+      <c r="C89" s="57"/>
       <c r="D89" s="9" t="s">
         <v>101</v>
       </c>
@@ -3901,14 +4439,14 @@
         <v>9</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="77.25" customHeight="1">
+    <row r="90" spans="1:7" ht="77.25" customHeight="1">
       <c r="A90" s="12">
         <v>85</v>
       </c>
-      <c r="B90" s="57">
+      <c r="B90" s="56">
         <v>46288</v>
       </c>
-      <c r="C90" s="56" t="s">
+      <c r="C90" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D90" s="12" t="s">
@@ -3921,12 +4459,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:7">
       <c r="A91" s="15">
         <v>86</v>
       </c>
-      <c r="B91" s="57"/>
-      <c r="C91" s="56"/>
+      <c r="B91" s="56"/>
+      <c r="C91" s="55"/>
       <c r="D91" s="15" t="s">
         <v>101</v>
       </c>
@@ -3937,12 +4475,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:7">
       <c r="A92" s="18">
         <v>87</v>
       </c>
-      <c r="B92" s="57"/>
-      <c r="C92" s="56"/>
+      <c r="B92" s="56"/>
+      <c r="C92" s="55"/>
       <c r="D92" s="15" t="s">
         <v>117</v>
       </c>
@@ -3953,12 +4491,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:7">
       <c r="A93" s="19">
         <v>88</v>
       </c>
-      <c r="B93" s="57"/>
-      <c r="C93" s="56"/>
+      <c r="B93" s="56"/>
+      <c r="C93" s="55"/>
       <c r="D93" s="15" t="s">
         <v>100</v>
       </c>
@@ -3969,12 +4507,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:7">
       <c r="A94" s="20">
         <v>89</v>
       </c>
-      <c r="B94" s="57"/>
-      <c r="C94" s="56"/>
+      <c r="B94" s="56"/>
+      <c r="C94" s="55"/>
       <c r="D94" s="15" t="s">
         <v>101</v>
       </c>
@@ -3985,24 +4523,24 @@
         <v>9</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:7">
       <c r="A95" s="20">
         <v>90</v>
       </c>
-      <c r="B95" s="57"/>
+      <c r="B95" s="56"/>
       <c r="C95" s="17"/>
       <c r="D95" s="17"/>
       <c r="E95" s="17"/>
       <c r="F95" s="17"/>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:7">
       <c r="A96" s="23">
         <v>91</v>
       </c>
-      <c r="B96" s="59">
+      <c r="B96" s="64">
         <v>46289</v>
       </c>
-      <c r="C96" s="60" t="s">
+      <c r="C96" s="65" t="s">
         <v>14</v>
       </c>
       <c r="D96" s="24" t="s">
@@ -4012,643 +4550,695 @@
         <v>120</v>
       </c>
       <c r="F96" s="22"/>
-    </row>
-    <row r="97" spans="1:6" ht="60">
+      <c r="G96" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="60">
       <c r="A97" s="23">
         <v>92</v>
       </c>
-      <c r="B97" s="59"/>
-      <c r="C97" s="60"/>
+      <c r="B97" s="64"/>
+      <c r="C97" s="65"/>
       <c r="D97" s="24" t="s">
         <v>99</v>
       </c>
       <c r="E97" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="F97" s="22"/>
-    </row>
-    <row r="98" spans="1:6" ht="60">
+      <c r="F97" s="22" t="s">
+        <v>199</v>
+      </c>
+      <c r="G97" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="60">
       <c r="A98" s="23">
         <v>93</v>
       </c>
-      <c r="B98" s="59"/>
-      <c r="C98" s="60"/>
+      <c r="B98" s="64"/>
+      <c r="C98" s="65"/>
       <c r="D98" s="24" t="s">
         <v>99</v>
       </c>
       <c r="E98" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="F98" s="22"/>
-    </row>
-    <row r="99" spans="1:6" ht="30">
+      <c r="F98" s="22" t="s">
+        <v>200</v>
+      </c>
+      <c r="G98" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="60">
       <c r="A99" s="23">
         <v>94</v>
       </c>
-      <c r="B99" s="59"/>
-      <c r="C99" s="60"/>
+      <c r="B99" s="64"/>
+      <c r="C99" s="65"/>
       <c r="D99" s="24" t="s">
         <v>99</v>
       </c>
       <c r="E99" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="F99" s="22"/>
-    </row>
-    <row r="100" spans="1:6">
+        <v>201</v>
+      </c>
+      <c r="F99" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="G99" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7">
       <c r="A100" s="23">
         <v>95</v>
       </c>
-      <c r="B100" s="59"/>
-      <c r="C100" s="60"/>
+      <c r="B100" s="64"/>
+      <c r="C100" s="65"/>
       <c r="D100" s="24" t="s">
         <v>109</v>
       </c>
       <c r="E100" s="28" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="F100" s="22"/>
     </row>
-    <row r="101" spans="1:6" ht="30">
+    <row r="101" spans="1:7" ht="30">
       <c r="A101" s="23">
         <v>96</v>
       </c>
-      <c r="B101" s="59"/>
-      <c r="C101" s="60"/>
+      <c r="B101" s="64"/>
+      <c r="C101" s="65"/>
       <c r="D101" s="24" t="s">
         <v>99</v>
       </c>
       <c r="E101" s="25" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F101" s="22"/>
-    </row>
-    <row r="102" spans="1:6" ht="45">
+      <c r="G101" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" ht="45">
       <c r="A102" s="23">
         <v>97</v>
       </c>
-      <c r="B102" s="59"/>
-      <c r="C102" s="60"/>
+      <c r="B102" s="64"/>
+      <c r="C102" s="65"/>
       <c r="D102" s="24" t="s">
         <v>109</v>
       </c>
       <c r="E102" s="27" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F102" s="22"/>
-    </row>
-    <row r="103" spans="1:6">
+      <c r="G102" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7">
       <c r="A103" s="23">
         <v>98</v>
       </c>
-      <c r="B103" s="59"/>
-      <c r="C103" s="60"/>
+      <c r="B103" s="64"/>
+      <c r="C103" s="65"/>
       <c r="D103" s="22"/>
       <c r="E103" s="22"/>
       <c r="F103" s="22"/>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:7">
       <c r="A104" s="23">
         <v>99</v>
       </c>
-      <c r="B104" s="59"/>
-      <c r="C104" s="60"/>
+      <c r="B104" s="64"/>
+      <c r="C104" s="65"/>
       <c r="D104" s="24" t="s">
         <v>109</v>
       </c>
       <c r="E104" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="F104" s="22"/>
-    </row>
-    <row r="105" spans="1:6">
+        <v>126</v>
+      </c>
+      <c r="F104" s="26" t="s">
+        <v>205</v>
+      </c>
+      <c r="G104" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7">
       <c r="A105" s="23">
         <v>100</v>
       </c>
-      <c r="B105" s="59"/>
-      <c r="C105" s="60"/>
+      <c r="B105" s="64"/>
+      <c r="C105" s="65"/>
       <c r="D105" s="24" t="s">
         <v>106</v>
       </c>
       <c r="E105" s="22" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F105" s="22"/>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:7">
       <c r="A106" s="23">
         <v>101</v>
       </c>
-      <c r="B106" s="59"/>
-      <c r="C106" s="60"/>
+      <c r="B106" s="64"/>
+      <c r="C106" s="65"/>
       <c r="D106" s="24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E106" s="22" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F106" s="22"/>
-    </row>
-    <row r="107" spans="1:6" ht="45">
+      <c r="G106" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="45">
       <c r="A107" s="23">
         <v>102</v>
       </c>
-      <c r="B107" s="59"/>
-      <c r="C107" s="60"/>
+      <c r="B107" s="64"/>
+      <c r="C107" s="65"/>
       <c r="D107" s="24" t="s">
         <v>101</v>
       </c>
       <c r="E107" s="26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F107" s="22"/>
-    </row>
-    <row r="108" spans="1:6" ht="45">
+      <c r="G107" s="38" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="45">
       <c r="A108" s="23">
         <v>103</v>
       </c>
-      <c r="B108" s="59"/>
-      <c r="C108" s="60"/>
+      <c r="B108" s="64"/>
+      <c r="C108" s="65"/>
       <c r="D108" s="24" t="s">
         <v>99</v>
       </c>
       <c r="E108" s="26" t="s">
-        <v>132</v>
+        <v>208</v>
       </c>
       <c r="F108" s="22"/>
-    </row>
-    <row r="109" spans="1:6">
+      <c r="G108" s="38" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7">
       <c r="A109" s="23">
         <v>104</v>
       </c>
-      <c r="B109" s="59"/>
-      <c r="C109" s="60"/>
+      <c r="B109" s="64"/>
+      <c r="C109" s="65"/>
       <c r="D109" s="24" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E109" s="22" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F109" s="22"/>
     </row>
-    <row r="110" spans="1:6" ht="45">
+    <row r="110" spans="1:7" ht="45">
       <c r="A110" s="23">
         <v>105</v>
       </c>
-      <c r="B110" s="50">
+      <c r="B110" s="61">
         <v>46290</v>
       </c>
-      <c r="C110" s="53" t="s">
+      <c r="C110" s="58" t="s">
         <v>39</v>
       </c>
       <c r="D110" s="15" t="s">
         <v>99</v>
       </c>
       <c r="E110" s="32" t="s">
-        <v>135</v>
-      </c>
-      <c r="F110" s="31"/>
-    </row>
-    <row r="111" spans="1:6" ht="45">
+        <v>212</v>
+      </c>
+      <c r="F110" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="G110" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" ht="45">
       <c r="A111" s="31"/>
-      <c r="B111" s="51"/>
-      <c r="C111" s="54"/>
+      <c r="B111" s="62"/>
+      <c r="C111" s="59"/>
       <c r="D111" s="24" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E111" s="32" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F111" s="31"/>
-    </row>
-    <row r="112" spans="1:6">
+      <c r="G111" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7">
       <c r="A112" s="31"/>
-      <c r="B112" s="51"/>
-      <c r="C112" s="54"/>
+      <c r="B112" s="62"/>
+      <c r="C112" s="59"/>
       <c r="D112" s="31"/>
       <c r="E112" s="31"/>
       <c r="F112" s="31"/>
+      <c r="G112" t="s">
+        <v>213</v>
+      </c>
     </row>
     <row r="113" spans="1:6" ht="45">
       <c r="A113" s="31"/>
-      <c r="B113" s="51"/>
-      <c r="C113" s="54"/>
+      <c r="B113" s="62"/>
+      <c r="C113" s="59"/>
       <c r="D113" s="31" t="s">
         <v>101</v>
       </c>
       <c r="E113" s="32" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F113" s="31"/>
     </row>
     <row r="114" spans="1:6" ht="60">
       <c r="A114" s="31"/>
-      <c r="B114" s="51"/>
-      <c r="C114" s="54"/>
+      <c r="B114" s="62"/>
+      <c r="C114" s="59"/>
       <c r="D114" s="31" t="s">
         <v>101</v>
       </c>
       <c r="E114" s="33" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F114" s="31"/>
     </row>
     <row r="115" spans="1:6" ht="75">
       <c r="A115" s="31"/>
-      <c r="B115" s="51"/>
-      <c r="C115" s="54"/>
+      <c r="B115" s="62"/>
+      <c r="C115" s="59"/>
       <c r="D115" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="E115" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="F115" s="31" t="s">
         <v>140</v>
-      </c>
-      <c r="E115" s="32" t="s">
-        <v>142</v>
-      </c>
-      <c r="F115" s="31" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" s="31"/>
-      <c r="B116" s="51"/>
-      <c r="C116" s="54"/>
+      <c r="B116" s="62"/>
+      <c r="C116" s="59"/>
       <c r="D116" s="31" t="s">
         <v>109</v>
       </c>
       <c r="E116" s="32" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F116" s="31"/>
     </row>
     <row r="117" spans="1:6" ht="45">
       <c r="A117" s="31"/>
-      <c r="B117" s="51"/>
-      <c r="C117" s="54"/>
+      <c r="B117" s="62"/>
+      <c r="C117" s="59"/>
       <c r="D117" s="31"/>
       <c r="E117" s="32" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="F117" s="31" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="118" spans="1:6">
       <c r="A118" s="31"/>
-      <c r="B118" s="51"/>
-      <c r="C118" s="54"/>
+      <c r="B118" s="62"/>
+      <c r="C118" s="59"/>
       <c r="D118" s="31"/>
       <c r="E118" s="31"/>
       <c r="F118" s="31"/>
     </row>
     <row r="119" spans="1:6" ht="30">
       <c r="A119" s="31"/>
-      <c r="B119" s="51"/>
-      <c r="C119" s="54"/>
+      <c r="B119" s="62"/>
+      <c r="C119" s="59"/>
       <c r="D119" s="31"/>
       <c r="E119" s="33" t="s">
+        <v>142</v>
+      </c>
+      <c r="F119" s="31" t="s">
         <v>145</v>
-      </c>
-      <c r="F119" s="31" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="75">
       <c r="A120" s="31"/>
-      <c r="B120" s="51"/>
-      <c r="C120" s="54"/>
+      <c r="B120" s="62"/>
+      <c r="C120" s="59"/>
       <c r="D120" s="31" t="s">
         <v>109</v>
       </c>
       <c r="E120" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="F120" s="32" t="s">
         <v>146</v>
-      </c>
-      <c r="F120" s="32" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="45">
       <c r="A121" s="31"/>
-      <c r="B121" s="52"/>
-      <c r="C121" s="55"/>
+      <c r="B121" s="63"/>
+      <c r="C121" s="60"/>
       <c r="D121" s="31" t="s">
         <v>109</v>
       </c>
       <c r="E121" s="32" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="F121" s="31"/>
     </row>
     <row r="122" spans="1:6" ht="30">
       <c r="A122" s="34"/>
-      <c r="B122" s="37">
+      <c r="B122" s="66">
         <v>46293</v>
       </c>
-      <c r="C122" s="40" t="s">
+      <c r="C122" s="77" t="s">
         <v>44</v>
       </c>
       <c r="D122" s="34" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E122" s="35" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F122" s="34"/>
     </row>
     <row r="123" spans="1:6" ht="75">
       <c r="A123" s="34"/>
-      <c r="B123" s="38"/>
-      <c r="C123" s="41"/>
+      <c r="B123" s="67"/>
+      <c r="C123" s="78"/>
       <c r="D123" s="34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="E123" s="36" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="F123" s="34"/>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" s="34"/>
-      <c r="B124" s="38"/>
-      <c r="C124" s="41"/>
+      <c r="B124" s="67"/>
+      <c r="C124" s="78"/>
       <c r="D124" s="34" t="s">
         <v>102</v>
       </c>
       <c r="E124" s="36" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F124" s="34"/>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" s="34"/>
-      <c r="B125" s="38"/>
-      <c r="C125" s="41"/>
+      <c r="B125" s="67"/>
+      <c r="C125" s="78"/>
       <c r="D125" s="34" t="s">
         <v>117</v>
       </c>
       <c r="E125" s="36" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="F125" s="34"/>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" s="34"/>
-      <c r="B126" s="38"/>
-      <c r="C126" s="41"/>
+      <c r="B126" s="67"/>
+      <c r="C126" s="78"/>
       <c r="D126" s="34" t="s">
         <v>117</v>
       </c>
       <c r="E126" s="36" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F126" s="34"/>
     </row>
     <row r="127" spans="1:6">
       <c r="A127" s="34"/>
-      <c r="B127" s="38"/>
-      <c r="C127" s="41"/>
+      <c r="B127" s="67"/>
+      <c r="C127" s="78"/>
       <c r="D127" s="34"/>
       <c r="E127" s="34"/>
       <c r="F127" s="34"/>
     </row>
     <row r="128" spans="1:6">
       <c r="A128" s="34"/>
-      <c r="B128" s="38"/>
-      <c r="C128" s="41"/>
+      <c r="B128" s="67"/>
+      <c r="C128" s="78"/>
       <c r="D128" s="34"/>
       <c r="E128" s="34"/>
       <c r="F128" s="34"/>
     </row>
     <row r="129" spans="1:8" ht="165">
       <c r="A129" s="34"/>
-      <c r="B129" s="38"/>
-      <c r="C129" s="41"/>
+      <c r="B129" s="67"/>
+      <c r="C129" s="78"/>
       <c r="D129" s="34"/>
       <c r="E129" s="35" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F129" s="36" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="60">
       <c r="A130" s="34"/>
-      <c r="B130" s="38"/>
-      <c r="C130" s="41"/>
+      <c r="B130" s="67"/>
+      <c r="C130" s="78"/>
       <c r="D130" s="34"/>
       <c r="E130" s="36" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="F130" s="34"/>
     </row>
     <row r="131" spans="1:8">
       <c r="A131" s="34"/>
-      <c r="B131" s="38"/>
-      <c r="C131" s="41"/>
+      <c r="B131" s="67"/>
+      <c r="C131" s="78"/>
       <c r="D131" s="34" t="s">
         <v>101</v>
       </c>
       <c r="E131" s="34" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F131" s="34"/>
     </row>
     <row r="132" spans="1:8">
       <c r="A132" s="34"/>
-      <c r="B132" s="38"/>
-      <c r="C132" s="41"/>
+      <c r="B132" s="67"/>
+      <c r="C132" s="78"/>
       <c r="D132" s="34" t="s">
         <v>101</v>
       </c>
       <c r="E132" s="34" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="F132" s="34"/>
     </row>
     <row r="133" spans="1:8">
       <c r="A133" s="34"/>
-      <c r="B133" s="38"/>
-      <c r="C133" s="41"/>
+      <c r="B133" s="67"/>
+      <c r="C133" s="78"/>
       <c r="D133" s="34"/>
       <c r="E133" s="34" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="F133" s="34"/>
     </row>
     <row r="134" spans="1:8" ht="45">
       <c r="A134" s="34"/>
-      <c r="B134" s="38"/>
-      <c r="C134" s="41"/>
+      <c r="B134" s="67"/>
+      <c r="C134" s="78"/>
       <c r="D134" s="34" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E134" s="36" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F134" s="34"/>
     </row>
     <row r="135" spans="1:8">
       <c r="A135" s="34"/>
-      <c r="B135" s="38"/>
-      <c r="C135" s="41"/>
+      <c r="B135" s="67"/>
+      <c r="C135" s="78"/>
       <c r="D135" s="34"/>
       <c r="E135" s="34"/>
       <c r="F135" s="34"/>
     </row>
     <row r="136" spans="1:8" ht="45">
       <c r="A136" s="34"/>
-      <c r="B136" s="38"/>
-      <c r="C136" s="41"/>
+      <c r="B136" s="67"/>
+      <c r="C136" s="78"/>
       <c r="D136" s="34"/>
       <c r="E136" s="36" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="F136" s="36" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="45">
       <c r="A137" s="34"/>
-      <c r="B137" s="39"/>
-      <c r="C137" s="42"/>
+      <c r="B137" s="68"/>
+      <c r="C137" s="79"/>
       <c r="D137" s="34"/>
       <c r="E137" s="35" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="F137" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="75">
       <c r="A138" s="31"/>
-      <c r="B138" s="50">
+      <c r="B138" s="61">
         <v>46295</v>
       </c>
-      <c r="C138" s="53" t="s">
+      <c r="C138" s="58" t="s">
         <v>7</v>
       </c>
       <c r="D138" s="31"/>
       <c r="E138" s="33" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="F138" s="32" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="139" spans="1:8" ht="60">
       <c r="A139" s="31"/>
-      <c r="B139" s="51"/>
-      <c r="C139" s="54"/>
+      <c r="B139" s="62"/>
+      <c r="C139" s="59"/>
       <c r="D139" s="31"/>
       <c r="E139" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="F139" s="32" t="s">
         <v>171</v>
-      </c>
-      <c r="F139" s="32" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="140" spans="1:8" ht="75">
       <c r="A140" s="31"/>
-      <c r="B140" s="51"/>
-      <c r="C140" s="54"/>
+      <c r="B140" s="62"/>
+      <c r="C140" s="59"/>
       <c r="D140" s="31"/>
       <c r="E140" s="33" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="F140" s="32" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="141" spans="1:8">
       <c r="A141" s="31"/>
-      <c r="B141" s="51"/>
-      <c r="C141" s="54"/>
+      <c r="B141" s="62"/>
+      <c r="C141" s="59"/>
       <c r="D141" s="31"/>
       <c r="E141" s="31"/>
       <c r="F141" s="31"/>
     </row>
     <row r="142" spans="1:8" ht="60">
       <c r="A142" s="31"/>
-      <c r="B142" s="51"/>
-      <c r="C142" s="54"/>
+      <c r="B142" s="62"/>
+      <c r="C142" s="59"/>
       <c r="D142" s="31"/>
       <c r="E142" s="33" t="s">
-        <v>175</v>
-      </c>
-      <c r="F142" s="61" t="s">
-        <v>179</v>
+        <v>172</v>
+      </c>
+      <c r="F142" s="37" t="s">
+        <v>176</v>
       </c>
       <c r="H142" s="21" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="143" spans="1:8" ht="75">
       <c r="A143" s="31"/>
-      <c r="B143" s="51"/>
-      <c r="C143" s="54"/>
+      <c r="B143" s="62"/>
+      <c r="C143" s="59"/>
       <c r="D143" s="31"/>
       <c r="E143" s="32" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="F143" s="32" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="144" spans="1:8">
       <c r="A144" s="31"/>
-      <c r="B144" s="51"/>
-      <c r="C144" s="54"/>
+      <c r="B144" s="62"/>
+      <c r="C144" s="59"/>
       <c r="D144" s="31"/>
       <c r="E144" s="31"/>
       <c r="F144" s="31"/>
     </row>
-    <row r="145" spans="1:8" ht="60">
+    <row r="145" spans="1:9" ht="60">
       <c r="A145" s="31"/>
-      <c r="B145" s="51"/>
-      <c r="C145" s="54"/>
+      <c r="B145" s="62"/>
+      <c r="C145" s="59"/>
       <c r="D145" s="31"/>
       <c r="E145" s="33" t="s">
-        <v>177</v>
-      </c>
-      <c r="F145" s="61" t="s">
-        <v>178</v>
+        <v>174</v>
+      </c>
+      <c r="F145" s="37" t="s">
+        <v>175</v>
       </c>
       <c r="H145" s="21" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="146" spans="1:8">
+        <v>179</v>
+      </c>
+      <c r="I145" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9">
       <c r="A146" s="31"/>
-      <c r="B146" s="52"/>
-      <c r="C146" s="55"/>
+      <c r="B146" s="63"/>
+      <c r="C146" s="60"/>
       <c r="D146" s="31" t="s">
         <v>102</v>
       </c>
       <c r="E146" s="31" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="F146" s="31"/>
     </row>
-    <row r="147" spans="1:8" ht="60">
+    <row r="147" spans="1:9" ht="60">
       <c r="B147" s="30">
         <v>46266</v>
       </c>
       <c r="D147" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E147" s="21" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="148" spans="1:8" ht="75">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" ht="75">
       <c r="E148" s="21" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="150" spans="1:8">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9">
       <c r="B150" s="30">
         <v>46270</v>
       </c>
     </row>
-    <row r="151" spans="1:8">
+    <row r="151" spans="1:9">
       <c r="B151" s="30">
         <v>46271</v>
       </c>
@@ -4656,118 +5246,527 @@
         <v>117</v>
       </c>
       <c r="E151" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" ht="45">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" ht="45">
       <c r="B152" s="30">
         <v>46271</v>
       </c>
       <c r="E152" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="F152" s="21" t="s">
+        <v>185</v>
+      </c>
+      <c r="H152" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" ht="45">
+      <c r="E153" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="F153" s="21" t="s">
         <v>187</v>
       </c>
-      <c r="F152" s="21" t="s">
+      <c r="H153" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" ht="75">
+      <c r="E154" s="21" t="s">
+        <v>193</v>
+      </c>
+      <c r="F154" s="21" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="153" spans="1:8" ht="45">
-      <c r="E153" s="21" t="s">
+      <c r="H154" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" ht="45">
+      <c r="E155" s="21" t="s">
         <v>189</v>
       </c>
-      <c r="F153" s="21" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="154" spans="1:8" ht="75">
-      <c r="E154" s="21" t="s">
-        <v>196</v>
-      </c>
-      <c r="F154" s="21" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="155" spans="1:8" ht="45">
-      <c r="E155" s="21" t="s">
-        <v>192</v>
-      </c>
       <c r="F155" s="21" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="156" spans="1:8" ht="45">
+        <v>187</v>
+      </c>
+      <c r="H155" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" ht="45">
       <c r="D156" t="s">
         <v>101</v>
       </c>
       <c r="E156" s="21" t="s">
+        <v>191</v>
+      </c>
+      <c r="F156" s="21" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" ht="30">
+      <c r="D157" t="s">
+        <v>101</v>
+      </c>
+      <c r="E157" s="21" t="s">
         <v>194</v>
       </c>
-      <c r="F156" s="21" t="s">
+      <c r="F157" s="21" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="157" spans="1:8" ht="30">
-      <c r="E157" s="21" t="s">
+      <c r="H157" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9">
+      <c r="A159" s="22"/>
+      <c r="B159" s="71">
+        <v>46302</v>
+      </c>
+      <c r="C159" s="74" t="s">
+        <v>215</v>
+      </c>
+      <c r="D159" s="22" t="s">
         <v>197</v>
       </c>
-      <c r="F157" s="21" t="s">
+      <c r="E159" s="26" t="s">
+        <v>196</v>
+      </c>
+      <c r="F159" s="22"/>
+    </row>
+    <row r="160" spans="1:9" ht="45">
+      <c r="A160" s="22"/>
+      <c r="B160" s="72"/>
+      <c r="C160" s="75"/>
+      <c r="D160" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="E160" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="F160" s="26" t="s">
         <v>198</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8" ht="45">
+      <c r="A161" s="22"/>
+      <c r="B161" s="72"/>
+      <c r="C161" s="75"/>
+      <c r="D161" s="22"/>
+      <c r="E161" s="26" t="s">
+        <v>203</v>
+      </c>
+      <c r="F161" s="26" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="162" spans="1:8" ht="90">
+      <c r="A162" s="22"/>
+      <c r="B162" s="72"/>
+      <c r="C162" s="75"/>
+      <c r="D162" s="22"/>
+      <c r="E162" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="F162" s="26" t="s">
+        <v>207</v>
+      </c>
+      <c r="H162" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" ht="60">
+      <c r="A163" s="22"/>
+      <c r="B163" s="72"/>
+      <c r="C163" s="75"/>
+      <c r="D163" s="22"/>
+      <c r="E163" s="26" t="s">
+        <v>210</v>
+      </c>
+      <c r="F163" s="26" t="s">
+        <v>211</v>
+      </c>
+      <c r="H163" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8">
+      <c r="A164" s="22"/>
+      <c r="B164" s="73"/>
+      <c r="C164" s="76"/>
+      <c r="D164" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="E164" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="F164" s="22"/>
+    </row>
+    <row r="165" spans="1:8">
+      <c r="B165" s="30">
+        <v>46303</v>
+      </c>
+      <c r="E165" s="39" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="167" spans="1:8" ht="45">
+      <c r="A167" s="41"/>
+      <c r="B167" s="42">
+        <v>46304</v>
+      </c>
+      <c r="C167" s="41"/>
+      <c r="D167" s="41" t="s">
+        <v>221</v>
+      </c>
+      <c r="E167" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="F167" s="43" t="s">
+        <v>187</v>
+      </c>
+      <c r="G167" s="40"/>
+    </row>
+    <row r="168" spans="1:8">
+      <c r="A168" s="41"/>
+      <c r="B168" s="41"/>
+      <c r="C168" s="41"/>
+      <c r="D168" s="41" t="s">
+        <v>219</v>
+      </c>
+      <c r="E168" s="43" t="s">
+        <v>218</v>
+      </c>
+      <c r="F168" s="41"/>
+      <c r="G168" s="40"/>
+    </row>
+    <row r="169" spans="1:8">
+      <c r="A169" s="41"/>
+      <c r="B169" s="41"/>
+      <c r="C169" s="41"/>
+      <c r="D169" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="E169" s="43" t="s">
+        <v>220</v>
+      </c>
+      <c r="F169" s="41"/>
+      <c r="G169" s="40"/>
+    </row>
+    <row r="170" spans="1:8">
+      <c r="A170" s="41"/>
+      <c r="B170" s="41"/>
+      <c r="C170" s="41"/>
+      <c r="D170" s="41" t="s">
+        <v>219</v>
+      </c>
+      <c r="E170" s="43" t="s">
+        <v>222</v>
+      </c>
+      <c r="F170" s="41"/>
+      <c r="G170" s="40"/>
+    </row>
+    <row r="171" spans="1:8">
+      <c r="B171" s="30">
+        <v>46307</v>
+      </c>
+      <c r="D171" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="E171" s="44" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="172" spans="1:8">
+      <c r="D172" s="40" t="s">
+        <v>100</v>
+      </c>
+      <c r="E172" s="44" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="173" spans="1:8" ht="45">
+      <c r="E173" s="44" t="s">
+        <v>225</v>
+      </c>
+      <c r="F173" s="21" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="174" spans="1:8">
+      <c r="B174" s="30">
+        <v>46308</v>
+      </c>
+      <c r="D174" t="s">
+        <v>102</v>
+      </c>
+      <c r="E174" s="44" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="175" spans="1:8">
+      <c r="D175" t="s">
+        <v>227</v>
+      </c>
+      <c r="E175" s="44" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="176" spans="1:8">
+      <c r="D176" t="s">
+        <v>228</v>
+      </c>
+      <c r="E176" s="44" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="177" spans="2:7">
+      <c r="B177" s="30">
+        <v>46309</v>
+      </c>
+      <c r="E177" s="44" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="178" spans="2:7">
+      <c r="D178" t="s">
+        <v>233</v>
+      </c>
+      <c r="E178" s="44" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="179" spans="2:7">
+      <c r="E179" s="44" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="180" spans="2:7">
+      <c r="D180" t="s">
+        <v>99</v>
+      </c>
+      <c r="E180" s="44" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="181" spans="2:7" ht="60">
+      <c r="E181" s="44" t="s">
+        <v>235</v>
+      </c>
+      <c r="F181" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="G181" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="183" spans="2:7" ht="45">
+      <c r="E183" s="21" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="186" spans="2:7" ht="60">
+      <c r="B186" s="30">
+        <v>46310</v>
+      </c>
+      <c r="E186" s="21" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="187" spans="2:7" ht="75">
+      <c r="E187" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="F187" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="189" spans="2:7" ht="360">
+      <c r="E189" s="21" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="191" spans="2:7" ht="45">
+      <c r="E191" s="21" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="193" spans="2:5" ht="105">
+      <c r="E193" s="45" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="195" spans="2:5" ht="15.75">
+      <c r="B195" s="30">
+        <v>46311</v>
+      </c>
+      <c r="E195" s="49" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="197" spans="2:5" ht="23.25">
+      <c r="E197" s="46" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="199" spans="2:5" ht="60">
+      <c r="E199" s="21" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="201" spans="2:5" ht="15.75">
+      <c r="E201" s="50" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="202" spans="2:5">
+      <c r="E202" s="47"/>
+    </row>
+    <row r="203" spans="2:5">
+      <c r="E203" s="48" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="204" spans="2:5">
+      <c r="E204" s="47"/>
+    </row>
+    <row r="205" spans="2:5">
+      <c r="E205" s="48" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="206" spans="2:5">
+      <c r="E206" s="47"/>
+    </row>
+    <row r="207" spans="2:5">
+      <c r="E207" s="48" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="208" spans="2:5">
+      <c r="E208" s="47"/>
+    </row>
+    <row r="209" spans="5:5">
+      <c r="E209" s="48" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="210" spans="5:5">
+      <c r="E210" s="47"/>
+    </row>
+    <row r="211" spans="5:5">
+      <c r="E211" s="48" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="213" spans="5:5" ht="45">
+      <c r="E213" s="21" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="215" spans="5:5" ht="23.25">
+      <c r="E215" s="46" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="217" spans="5:5" ht="60">
+      <c r="E217" s="21" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="219" spans="5:5" ht="30">
+      <c r="E219" s="21" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="221" spans="5:5" ht="23.25">
+      <c r="E221" s="46" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="223" spans="5:5" ht="60">
+      <c r="E223" s="21" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="225" spans="2:5" ht="23.25">
+      <c r="E225" s="46" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="227" spans="2:5" ht="45">
+      <c r="E227" s="21" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="229" spans="2:5">
+      <c r="B229" s="30">
+        <v>46317</v>
+      </c>
+      <c r="E229" t="s">
+        <v>262</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:F90" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
-  <mergeCells count="52">
+  <mergeCells count="54">
+    <mergeCell ref="D71:D77"/>
+    <mergeCell ref="B39:B45"/>
+    <mergeCell ref="C39:C45"/>
+    <mergeCell ref="D39:D45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="C34:C38"/>
+    <mergeCell ref="D34:D38"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="B159:B164"/>
+    <mergeCell ref="C159:C164"/>
+    <mergeCell ref="C122:C137"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="D3:D7"/>
+    <mergeCell ref="B8:B16"/>
+    <mergeCell ref="C8:C16"/>
     <mergeCell ref="C138:C146"/>
     <mergeCell ref="B138:B146"/>
     <mergeCell ref="B110:B121"/>
     <mergeCell ref="C110:C121"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="B96:B109"/>
+    <mergeCell ref="C96:C109"/>
+    <mergeCell ref="B122:B137"/>
     <mergeCell ref="C90:C94"/>
     <mergeCell ref="B90:B95"/>
     <mergeCell ref="B78:B83"/>
     <mergeCell ref="C78:C83"/>
     <mergeCell ref="B84:B89"/>
     <mergeCell ref="C84:C89"/>
-    <mergeCell ref="B96:B109"/>
-    <mergeCell ref="C96:C109"/>
-    <mergeCell ref="C39:C45"/>
-    <mergeCell ref="D39:D45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="D71:D77"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="C67:C70"/>
+    <mergeCell ref="B71:B77"/>
+    <mergeCell ref="C71:C77"/>
     <mergeCell ref="B52:B57"/>
     <mergeCell ref="C52:C57"/>
     <mergeCell ref="B58:B61"/>
     <mergeCell ref="C58:C61"/>
     <mergeCell ref="B62:B66"/>
     <mergeCell ref="C62:C66"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="C67:C70"/>
-    <mergeCell ref="B71:B77"/>
-    <mergeCell ref="C71:C77"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="D3:D7"/>
-    <mergeCell ref="B8:B16"/>
-    <mergeCell ref="C8:C16"/>
-    <mergeCell ref="B122:B137"/>
-    <mergeCell ref="C122:C137"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="B21:B25"/>
-    <mergeCell ref="C21:C25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="B39:B45"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>

<commit_message>
worked on apiclient issue-Laxmi27-10-2026
</commit_message>
<xml_diff>
--- a/Action_Items_Tracking_Sheet_Formatted.xlsx
+++ b/Action_Items_Tracking_Sheet_Formatted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AITO-Recovered\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEF0EA5E-501C-420F-8E62-C4B05873ADD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A74DA8D8-91F9-49DA-ACF5-7E044B7AFB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="268">
   <si>
     <t>Action Items &amp; Work Hours Tracking Log</t>
   </si>
@@ -2235,6 +2235,12 @@
   </si>
   <si>
     <t>3hr 30 mi</t>
+  </si>
+  <si>
+    <t>Revised claude workshop concepts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">worked on merge conflicts and shared new  updated zip file </t>
   </si>
 </sst>
 </file>
@@ -2655,24 +2661,27 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2700,9 +2709,6 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2742,7 +2748,7 @@
     <xf numFmtId="164" fontId="3" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3012,7 +3018,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I231"/>
+  <dimension ref="A1:I234"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -3025,14 +3031,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1">
-      <c r="A1" s="66" t="s">
+      <c r="A1" s="56" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="66"/>
-      <c r="D1" s="66"/>
-      <c r="E1" s="66"/>
-      <c r="F1" s="66"/>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+      <c r="F1" s="56"/>
     </row>
     <row r="2" spans="1:6" ht="21.75" customHeight="1">
       <c r="A2" s="3" t="s">
@@ -3058,13 +3064,13 @@
       <c r="A3" s="2">
         <v>1</v>
       </c>
-      <c r="B3" s="52">
+      <c r="B3" s="53">
         <v>46260</v>
       </c>
-      <c r="C3" s="56" t="s">
+      <c r="C3" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="51">
+      <c r="D3" s="57">
         <v>6.5</v>
       </c>
       <c r="E3" s="4" t="s">
@@ -3078,9 +3084,9 @@
       <c r="A4" s="2">
         <v>2</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="53"/>
       <c r="E4" s="4" t="s">
         <v>10</v>
       </c>
@@ -3092,9 +3098,9 @@
       <c r="A5" s="2">
         <v>3</v>
       </c>
-      <c r="B5" s="52"/>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="53"/>
       <c r="E5" s="4" t="s">
         <v>11</v>
       </c>
@@ -3106,9 +3112,9 @@
       <c r="A6" s="2">
         <v>4</v>
       </c>
-      <c r="B6" s="52"/>
-      <c r="C6" s="52"/>
-      <c r="D6" s="52"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="53"/>
       <c r="E6" s="4" t="s">
         <v>12</v>
       </c>
@@ -3120,9 +3126,9 @@
       <c r="A7" s="2">
         <v>5</v>
       </c>
-      <c r="B7" s="52"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="52"/>
+      <c r="B7" s="53"/>
+      <c r="C7" s="53"/>
+      <c r="D7" s="53"/>
       <c r="E7" s="4" t="s">
         <v>13</v>
       </c>
@@ -3134,10 +3140,10 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="53">
+      <c r="B8" s="52">
         <v>46261</v>
       </c>
-      <c r="C8" s="54" t="s">
+      <c r="C8" s="51" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -3154,8 +3160,8 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="53"/>
-      <c r="C9" s="53"/>
+      <c r="B9" s="52"/>
+      <c r="C9" s="52"/>
       <c r="D9" s="1" t="s">
         <v>111</v>
       </c>
@@ -3170,8 +3176,8 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="53"/>
-      <c r="C10" s="53"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="52"/>
       <c r="D10" s="1" t="s">
         <v>99</v>
       </c>
@@ -3186,8 +3192,8 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="53"/>
-      <c r="C11" s="53"/>
+      <c r="B11" s="52"/>
+      <c r="C11" s="52"/>
       <c r="D11" s="1" t="s">
         <v>101</v>
       </c>
@@ -3202,8 +3208,8 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="53"/>
-      <c r="C12" s="53"/>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
       <c r="D12" s="1" t="s">
         <v>109</v>
       </c>
@@ -3218,8 +3224,8 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="53"/>
-      <c r="C13" s="53"/>
+      <c r="B13" s="52"/>
+      <c r="C13" s="52"/>
       <c r="D13" s="1" t="s">
         <v>109</v>
       </c>
@@ -3234,8 +3240,8 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="53"/>
-      <c r="C14" s="53"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="52"/>
       <c r="D14" s="1" t="s">
         <v>99</v>
       </c>
@@ -3250,8 +3256,8 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="53"/>
-      <c r="C15" s="53"/>
+      <c r="B15" s="52"/>
+      <c r="C15" s="52"/>
       <c r="D15" s="1" t="s">
         <v>101</v>
       </c>
@@ -3266,8 +3272,8 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="53"/>
-      <c r="C16" s="53"/>
+      <c r="B16" s="52"/>
+      <c r="C16" s="52"/>
       <c r="D16" s="1" t="s">
         <v>101</v>
       </c>
@@ -3282,10 +3288,10 @@
       <c r="A17" s="2">
         <v>15</v>
       </c>
-      <c r="B17" s="52">
+      <c r="B17" s="53">
         <v>46266</v>
       </c>
-      <c r="C17" s="56" t="s">
+      <c r="C17" s="55" t="s">
         <v>24</v>
       </c>
       <c r="D17" s="2" t="s">
@@ -3302,8 +3308,8 @@
       <c r="A18" s="2">
         <v>16</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="52"/>
+      <c r="B18" s="53"/>
+      <c r="C18" s="53"/>
       <c r="D18" s="2" t="s">
         <v>103</v>
       </c>
@@ -3318,8 +3324,8 @@
       <c r="A19" s="2">
         <v>17</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="52"/>
+      <c r="B19" s="53"/>
+      <c r="C19" s="53"/>
       <c r="D19" s="2" t="s">
         <v>101</v>
       </c>
@@ -3334,8 +3340,8 @@
       <c r="A20" s="2">
         <v>18</v>
       </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="52"/>
+      <c r="B20" s="53"/>
+      <c r="C20" s="53"/>
       <c r="D20" s="2" t="s">
         <v>112</v>
       </c>
@@ -3350,10 +3356,10 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="53">
+      <c r="B21" s="52">
         <v>46267</v>
       </c>
-      <c r="C21" s="54" t="s">
+      <c r="C21" s="51" t="s">
         <v>7</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -3370,8 +3376,8 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="53"/>
-      <c r="C22" s="53"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
       <c r="D22" s="1" t="s">
         <v>102</v>
       </c>
@@ -3386,8 +3392,8 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
+      <c r="B23" s="52"/>
+      <c r="C23" s="52"/>
       <c r="D23" s="1" t="s">
         <v>101</v>
       </c>
@@ -3402,8 +3408,8 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="53"/>
-      <c r="C24" s="53"/>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
       <c r="D24" s="1" t="s">
         <v>101</v>
       </c>
@@ -3418,8 +3424,8 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="53"/>
-      <c r="C25" s="53"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="52"/>
       <c r="D25" s="1" t="s">
         <v>101</v>
       </c>
@@ -3434,13 +3440,13 @@
       <c r="A26" s="2">
         <v>24</v>
       </c>
-      <c r="B26" s="52">
+      <c r="B26" s="53">
         <v>46268</v>
       </c>
-      <c r="C26" s="56" t="s">
+      <c r="C26" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="D26" s="51">
+      <c r="D26" s="57">
         <v>7</v>
       </c>
       <c r="E26" s="4" t="s">
@@ -3454,9 +3460,9 @@
       <c r="A27" s="2">
         <v>25</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="52"/>
-      <c r="D27" s="52"/>
+      <c r="B27" s="53"/>
+      <c r="C27" s="53"/>
+      <c r="D27" s="53"/>
       <c r="E27" s="4" t="s">
         <v>36</v>
       </c>
@@ -3468,9 +3474,9 @@
       <c r="A28" s="2">
         <v>26</v>
       </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="52"/>
-      <c r="D28" s="52"/>
+      <c r="B28" s="53"/>
+      <c r="C28" s="53"/>
+      <c r="D28" s="53"/>
       <c r="E28" s="4" t="s">
         <v>37</v>
       </c>
@@ -3482,9 +3488,9 @@
       <c r="A29" s="2">
         <v>27</v>
       </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
-      <c r="D29" s="52"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="53"/>
+      <c r="D29" s="53"/>
       <c r="E29" s="4" t="s">
         <v>38</v>
       </c>
@@ -3496,13 +3502,13 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="53">
+      <c r="B30" s="52">
         <v>46269</v>
       </c>
-      <c r="C30" s="54" t="s">
+      <c r="C30" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="D30" s="55">
+      <c r="D30" s="80">
         <v>7</v>
       </c>
       <c r="E30" s="6" t="s">
@@ -3516,9 +3522,9 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
+      <c r="B31" s="52"/>
+      <c r="C31" s="52"/>
+      <c r="D31" s="52"/>
       <c r="E31" s="6" t="s">
         <v>41</v>
       </c>
@@ -3530,9 +3536,9 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="53"/>
-      <c r="C32" s="53"/>
-      <c r="D32" s="53"/>
+      <c r="B32" s="52"/>
+      <c r="C32" s="52"/>
+      <c r="D32" s="52"/>
       <c r="E32" s="6" t="s">
         <v>42</v>
       </c>
@@ -3544,9 +3550,9 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="53"/>
-      <c r="C33" s="53"/>
-      <c r="D33" s="53"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="52"/>
+      <c r="D33" s="52"/>
       <c r="E33" s="6" t="s">
         <v>43</v>
       </c>
@@ -3558,13 +3564,13 @@
       <c r="A34" s="2">
         <v>32</v>
       </c>
-      <c r="B34" s="52">
+      <c r="B34" s="53">
         <v>46272</v>
       </c>
-      <c r="C34" s="56" t="s">
+      <c r="C34" s="55" t="s">
         <v>44</v>
       </c>
-      <c r="D34" s="51">
+      <c r="D34" s="57">
         <v>8</v>
       </c>
       <c r="E34" s="4" t="s">
@@ -3578,9 +3584,9 @@
       <c r="A35" s="2">
         <v>33</v>
       </c>
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
+      <c r="B35" s="53"/>
+      <c r="C35" s="53"/>
+      <c r="D35" s="53"/>
       <c r="E35" s="4" t="s">
         <v>46</v>
       </c>
@@ -3592,9 +3598,9 @@
       <c r="A36" s="2">
         <v>34</v>
       </c>
-      <c r="B36" s="52"/>
-      <c r="C36" s="52"/>
-      <c r="D36" s="52"/>
+      <c r="B36" s="53"/>
+      <c r="C36" s="53"/>
+      <c r="D36" s="53"/>
       <c r="E36" s="4" t="s">
         <v>47</v>
       </c>
@@ -3606,9 +3612,9 @@
       <c r="A37" s="2">
         <v>35</v>
       </c>
-      <c r="B37" s="52"/>
-      <c r="C37" s="52"/>
-      <c r="D37" s="52"/>
+      <c r="B37" s="53"/>
+      <c r="C37" s="53"/>
+      <c r="D37" s="53"/>
       <c r="E37" s="4" t="s">
         <v>48</v>
       </c>
@@ -3620,9 +3626,9 @@
       <c r="A38" s="2">
         <v>36</v>
       </c>
-      <c r="B38" s="52"/>
-      <c r="C38" s="52"/>
-      <c r="D38" s="52"/>
+      <c r="B38" s="53"/>
+      <c r="C38" s="53"/>
+      <c r="D38" s="53"/>
       <c r="E38" s="4" t="s">
         <v>49</v>
       </c>
@@ -3634,13 +3640,13 @@
       <c r="A39" s="1">
         <v>37</v>
       </c>
-      <c r="B39" s="53">
+      <c r="B39" s="52">
         <v>46273</v>
       </c>
-      <c r="C39" s="54" t="s">
+      <c r="C39" s="51" t="s">
         <v>24</v>
       </c>
-      <c r="D39" s="55">
+      <c r="D39" s="80">
         <v>6</v>
       </c>
       <c r="E39" s="6" t="s">
@@ -3654,9 +3660,9 @@
       <c r="A40" s="1">
         <v>38</v>
       </c>
-      <c r="B40" s="53"/>
-      <c r="C40" s="53"/>
-      <c r="D40" s="53"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="52"/>
+      <c r="D40" s="52"/>
       <c r="E40" s="6" t="s">
         <v>51</v>
       </c>
@@ -3668,9 +3674,9 @@
       <c r="A41" s="1">
         <v>39</v>
       </c>
-      <c r="B41" s="53"/>
-      <c r="C41" s="53"/>
-      <c r="D41" s="53"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="52"/>
+      <c r="D41" s="52"/>
       <c r="E41" s="6" t="s">
         <v>52</v>
       </c>
@@ -3682,9 +3688,9 @@
       <c r="A42" s="1">
         <v>40</v>
       </c>
-      <c r="B42" s="53"/>
-      <c r="C42" s="53"/>
-      <c r="D42" s="53"/>
+      <c r="B42" s="52"/>
+      <c r="C42" s="52"/>
+      <c r="D42" s="52"/>
       <c r="E42" s="6" t="s">
         <v>53</v>
       </c>
@@ -3696,9 +3702,9 @@
       <c r="A43" s="1">
         <v>41</v>
       </c>
-      <c r="B43" s="53"/>
-      <c r="C43" s="53"/>
-      <c r="D43" s="53"/>
+      <c r="B43" s="52"/>
+      <c r="C43" s="52"/>
+      <c r="D43" s="52"/>
       <c r="E43" s="6" t="s">
         <v>54</v>
       </c>
@@ -3710,9 +3716,9 @@
       <c r="A44" s="1">
         <v>42</v>
       </c>
-      <c r="B44" s="53"/>
-      <c r="C44" s="53"/>
-      <c r="D44" s="53"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="52"/>
+      <c r="D44" s="52"/>
       <c r="E44" s="6" t="s">
         <v>55</v>
       </c>
@@ -3724,9 +3730,9 @@
       <c r="A45" s="1">
         <v>43</v>
       </c>
-      <c r="B45" s="53"/>
-      <c r="C45" s="53"/>
-      <c r="D45" s="53"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="52"/>
       <c r="E45" s="6" t="s">
         <v>56</v>
       </c>
@@ -3738,10 +3744,10 @@
       <c r="A46" s="2">
         <v>44</v>
       </c>
-      <c r="B46" s="52">
+      <c r="B46" s="53">
         <v>46274</v>
       </c>
-      <c r="C46" s="56" t="s">
+      <c r="C46" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D46" s="2" t="s">
@@ -3758,8 +3764,8 @@
       <c r="A47" s="2">
         <v>45</v>
       </c>
-      <c r="B47" s="52"/>
-      <c r="C47" s="52"/>
+      <c r="B47" s="53"/>
+      <c r="C47" s="53"/>
       <c r="D47" s="2" t="s">
         <v>99</v>
       </c>
@@ -3772,8 +3778,8 @@
     </row>
     <row r="48" spans="1:6" ht="34.5" customHeight="1">
       <c r="A48" s="2"/>
-      <c r="B48" s="52"/>
-      <c r="C48" s="52"/>
+      <c r="B48" s="53"/>
+      <c r="C48" s="53"/>
       <c r="D48" s="2" t="s">
         <v>102</v>
       </c>
@@ -3786,8 +3792,8 @@
       <c r="A49" s="2">
         <v>46</v>
       </c>
-      <c r="B49" s="52"/>
-      <c r="C49" s="52"/>
+      <c r="B49" s="53"/>
+      <c r="C49" s="53"/>
       <c r="D49" s="2" t="s">
         <v>100</v>
       </c>
@@ -3799,13 +3805,13 @@
       </c>
     </row>
     <row r="50" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A50" s="54">
+      <c r="A50" s="51">
         <v>47</v>
       </c>
-      <c r="B50" s="53">
+      <c r="B50" s="52">
         <v>46275</v>
       </c>
-      <c r="C50" s="54" t="s">
+      <c r="C50" s="51" t="s">
         <v>14</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -3819,9 +3825,9 @@
       </c>
     </row>
     <row r="51" spans="1:6" ht="20.25" customHeight="1">
-      <c r="A51" s="54"/>
-      <c r="B51" s="54"/>
-      <c r="C51" s="54"/>
+      <c r="A51" s="51"/>
+      <c r="B51" s="51"/>
+      <c r="C51" s="51"/>
       <c r="D51" s="1" t="s">
         <v>100</v>
       </c>
@@ -3836,10 +3842,10 @@
       <c r="A52" s="2">
         <v>49</v>
       </c>
-      <c r="B52" s="52">
+      <c r="B52" s="53">
         <v>46276</v>
       </c>
-      <c r="C52" s="56" t="s">
+      <c r="C52" s="55" t="s">
         <v>39</v>
       </c>
       <c r="D52" s="2" t="s">
@@ -3856,8 +3862,8 @@
       <c r="A53" s="2">
         <v>50</v>
       </c>
-      <c r="B53" s="52"/>
-      <c r="C53" s="52"/>
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
       <c r="D53" s="2" t="s">
         <v>105</v>
       </c>
@@ -3872,8 +3878,8 @@
       <c r="A54" s="2">
         <v>51</v>
       </c>
-      <c r="B54" s="52"/>
-      <c r="C54" s="52"/>
+      <c r="B54" s="53"/>
+      <c r="C54" s="53"/>
       <c r="D54" s="2" t="s">
         <v>107</v>
       </c>
@@ -3888,8 +3894,8 @@
       <c r="A55" s="2">
         <v>52</v>
       </c>
-      <c r="B55" s="52"/>
-      <c r="C55" s="52"/>
+      <c r="B55" s="53"/>
+      <c r="C55" s="53"/>
       <c r="D55" s="2" t="s">
         <v>99</v>
       </c>
@@ -3902,8 +3908,8 @@
     </row>
     <row r="56" spans="1:6" ht="34.5" customHeight="1">
       <c r="A56" s="2"/>
-      <c r="B56" s="52"/>
-      <c r="C56" s="52"/>
+      <c r="B56" s="53"/>
+      <c r="C56" s="53"/>
       <c r="D56" s="2" t="s">
         <v>102</v>
       </c>
@@ -3916,8 +3922,8 @@
       <c r="A57" s="2">
         <v>53</v>
       </c>
-      <c r="B57" s="52"/>
-      <c r="C57" s="52"/>
+      <c r="B57" s="53"/>
+      <c r="C57" s="53"/>
       <c r="D57" s="2" t="s">
         <v>105</v>
       </c>
@@ -3932,10 +3938,10 @@
       <c r="A58" s="1">
         <v>54</v>
       </c>
-      <c r="B58" s="53">
+      <c r="B58" s="52">
         <v>46280</v>
       </c>
-      <c r="C58" s="54" t="s">
+      <c r="C58" s="51" t="s">
         <v>24</v>
       </c>
       <c r="D58" s="1" t="s">
@@ -3952,8 +3958,8 @@
       <c r="A59" s="1">
         <v>55</v>
       </c>
-      <c r="B59" s="53"/>
-      <c r="C59" s="53"/>
+      <c r="B59" s="52"/>
+      <c r="C59" s="52"/>
       <c r="D59" s="1" t="s">
         <v>102</v>
       </c>
@@ -3968,8 +3974,8 @@
       <c r="A60" s="1">
         <v>56</v>
       </c>
-      <c r="B60" s="53"/>
-      <c r="C60" s="53"/>
+      <c r="B60" s="52"/>
+      <c r="C60" s="52"/>
       <c r="D60" s="1" t="s">
         <v>105</v>
       </c>
@@ -3984,8 +3990,8 @@
       <c r="A61" s="1">
         <v>57</v>
       </c>
-      <c r="B61" s="53"/>
-      <c r="C61" s="53"/>
+      <c r="B61" s="52"/>
+      <c r="C61" s="52"/>
       <c r="D61" s="1" t="s">
         <v>106</v>
       </c>
@@ -4000,10 +4006,10 @@
       <c r="A62" s="2">
         <v>58</v>
       </c>
-      <c r="B62" s="52">
+      <c r="B62" s="53">
         <v>46281</v>
       </c>
-      <c r="C62" s="56" t="s">
+      <c r="C62" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D62" s="2" t="s">
@@ -4020,8 +4026,8 @@
       <c r="A63" s="2">
         <v>59</v>
       </c>
-      <c r="B63" s="52"/>
-      <c r="C63" s="52"/>
+      <c r="B63" s="53"/>
+      <c r="C63" s="53"/>
       <c r="D63" s="2" t="s">
         <v>102</v>
       </c>
@@ -4036,8 +4042,8 @@
       <c r="A64" s="2">
         <v>60</v>
       </c>
-      <c r="B64" s="52"/>
-      <c r="C64" s="52"/>
+      <c r="B64" s="53"/>
+      <c r="C64" s="53"/>
       <c r="D64" s="2" t="s">
         <v>101</v>
       </c>
@@ -4052,8 +4058,8 @@
       <c r="A65" s="2">
         <v>61</v>
       </c>
-      <c r="B65" s="52"/>
-      <c r="C65" s="52"/>
+      <c r="B65" s="53"/>
+      <c r="C65" s="53"/>
       <c r="D65" s="2" t="s">
         <v>101</v>
       </c>
@@ -4068,8 +4074,8 @@
       <c r="A66" s="2">
         <v>62</v>
       </c>
-      <c r="B66" s="52"/>
-      <c r="C66" s="52"/>
+      <c r="B66" s="53"/>
+      <c r="C66" s="53"/>
       <c r="D66" s="2" t="s">
         <v>102</v>
       </c>
@@ -4084,10 +4090,10 @@
       <c r="A67" s="1">
         <v>63</v>
       </c>
-      <c r="B67" s="53">
+      <c r="B67" s="52">
         <v>46282</v>
       </c>
-      <c r="C67" s="54" t="s">
+      <c r="C67" s="51" t="s">
         <v>14</v>
       </c>
       <c r="D67" s="1" t="s">
@@ -4104,8 +4110,8 @@
       <c r="A68" s="1">
         <v>64</v>
       </c>
-      <c r="B68" s="53"/>
-      <c r="C68" s="53"/>
+      <c r="B68" s="52"/>
+      <c r="C68" s="52"/>
       <c r="D68" s="1" t="s">
         <v>105</v>
       </c>
@@ -4120,8 +4126,8 @@
       <c r="A69" s="1">
         <v>65</v>
       </c>
-      <c r="B69" s="53"/>
-      <c r="C69" s="53"/>
+      <c r="B69" s="52"/>
+      <c r="C69" s="52"/>
       <c r="D69" s="1" t="s">
         <v>102</v>
       </c>
@@ -4136,8 +4142,8 @@
       <c r="A70" s="1">
         <v>66</v>
       </c>
-      <c r="B70" s="53"/>
-      <c r="C70" s="53"/>
+      <c r="B70" s="52"/>
+      <c r="C70" s="52"/>
       <c r="D70" s="1" t="s">
         <v>104</v>
       </c>
@@ -4152,13 +4158,13 @@
       <c r="A71" s="2">
         <v>67</v>
       </c>
-      <c r="B71" s="52">
+      <c r="B71" s="53">
         <v>46283</v>
       </c>
-      <c r="C71" s="56" t="s">
+      <c r="C71" s="55" t="s">
         <v>39</v>
       </c>
-      <c r="D71" s="51">
+      <c r="D71" s="57">
         <v>7</v>
       </c>
       <c r="E71" s="4" t="s">
@@ -4172,9 +4178,9 @@
       <c r="A72" s="2">
         <v>68</v>
       </c>
-      <c r="B72" s="52"/>
-      <c r="C72" s="52"/>
-      <c r="D72" s="52"/>
+      <c r="B72" s="53"/>
+      <c r="C72" s="53"/>
+      <c r="D72" s="53"/>
       <c r="E72" s="4" t="s">
         <v>82</v>
       </c>
@@ -4186,9 +4192,9 @@
       <c r="A73" s="2">
         <v>69</v>
       </c>
-      <c r="B73" s="52"/>
-      <c r="C73" s="52"/>
-      <c r="D73" s="52"/>
+      <c r="B73" s="53"/>
+      <c r="C73" s="53"/>
+      <c r="D73" s="53"/>
       <c r="E73" s="4" t="s">
         <v>83</v>
       </c>
@@ -4200,9 +4206,9 @@
       <c r="A74" s="2">
         <v>70</v>
       </c>
-      <c r="B74" s="52"/>
-      <c r="C74" s="52"/>
-      <c r="D74" s="52"/>
+      <c r="B74" s="53"/>
+      <c r="C74" s="53"/>
+      <c r="D74" s="53"/>
       <c r="E74" s="4" t="s">
         <v>84</v>
       </c>
@@ -4214,9 +4220,9 @@
       <c r="A75" s="2">
         <v>71</v>
       </c>
-      <c r="B75" s="52"/>
-      <c r="C75" s="52"/>
-      <c r="D75" s="52"/>
+      <c r="B75" s="53"/>
+      <c r="C75" s="53"/>
+      <c r="D75" s="53"/>
       <c r="E75" s="4" t="s">
         <v>85</v>
       </c>
@@ -4228,9 +4234,9 @@
       <c r="A76" s="2">
         <v>72</v>
       </c>
-      <c r="B76" s="52"/>
-      <c r="C76" s="52"/>
-      <c r="D76" s="52"/>
+      <c r="B76" s="53"/>
+      <c r="C76" s="53"/>
+      <c r="D76" s="53"/>
       <c r="E76" s="4" t="s">
         <v>86</v>
       </c>
@@ -4242,9 +4248,9 @@
       <c r="A77" s="2">
         <v>73</v>
       </c>
-      <c r="B77" s="52"/>
-      <c r="C77" s="52"/>
-      <c r="D77" s="52"/>
+      <c r="B77" s="53"/>
+      <c r="C77" s="53"/>
+      <c r="D77" s="53"/>
       <c r="E77" s="4" t="s">
         <v>87</v>
       </c>
@@ -4256,10 +4262,10 @@
       <c r="A78" s="1">
         <v>74</v>
       </c>
-      <c r="B78" s="53">
+      <c r="B78" s="52">
         <v>46286</v>
       </c>
-      <c r="C78" s="54" t="s">
+      <c r="C78" s="51" t="s">
         <v>44</v>
       </c>
       <c r="D78" s="1" t="s">
@@ -4276,8 +4282,8 @@
       <c r="A79" s="1">
         <v>75</v>
       </c>
-      <c r="B79" s="53"/>
-      <c r="C79" s="53"/>
+      <c r="B79" s="52"/>
+      <c r="C79" s="52"/>
       <c r="D79" s="1" t="s">
         <v>102</v>
       </c>
@@ -4292,8 +4298,8 @@
       <c r="A80" s="1">
         <v>76</v>
       </c>
-      <c r="B80" s="53"/>
-      <c r="C80" s="53"/>
+      <c r="B80" s="52"/>
+      <c r="C80" s="52"/>
       <c r="D80" s="1" t="s">
         <v>103</v>
       </c>
@@ -4308,8 +4314,8 @@
       <c r="A81" s="1">
         <v>77</v>
       </c>
-      <c r="B81" s="53"/>
-      <c r="C81" s="53"/>
+      <c r="B81" s="52"/>
+      <c r="C81" s="52"/>
       <c r="D81" s="1" t="s">
         <v>102</v>
       </c>
@@ -4324,8 +4330,8 @@
       <c r="A82" s="1">
         <v>78</v>
       </c>
-      <c r="B82" s="53"/>
-      <c r="C82" s="53"/>
+      <c r="B82" s="52"/>
+      <c r="C82" s="52"/>
       <c r="D82" s="1" t="s">
         <v>101</v>
       </c>
@@ -4340,8 +4346,8 @@
       <c r="A83" s="1">
         <v>79</v>
       </c>
-      <c r="B83" s="53"/>
-      <c r="C83" s="53"/>
+      <c r="B83" s="52"/>
+      <c r="C83" s="52"/>
       <c r="D83" s="1" t="s">
         <v>102</v>
       </c>
@@ -4356,10 +4362,10 @@
       <c r="A84" s="2">
         <v>80</v>
       </c>
-      <c r="B84" s="52">
+      <c r="B84" s="53">
         <v>46287</v>
       </c>
-      <c r="C84" s="56" t="s">
+      <c r="C84" s="55" t="s">
         <v>24</v>
       </c>
       <c r="D84" s="2" t="s">
@@ -4376,8 +4382,8 @@
       <c r="A85" s="2">
         <v>81</v>
       </c>
-      <c r="B85" s="52"/>
-      <c r="C85" s="52"/>
+      <c r="B85" s="53"/>
+      <c r="C85" s="53"/>
       <c r="D85" s="2" t="s">
         <v>99</v>
       </c>
@@ -4392,8 +4398,8 @@
       <c r="A86" s="2">
         <v>82</v>
       </c>
-      <c r="B86" s="52"/>
-      <c r="C86" s="52"/>
+      <c r="B86" s="53"/>
+      <c r="C86" s="53"/>
       <c r="D86" s="2" t="s">
         <v>100</v>
       </c>
@@ -4408,8 +4414,8 @@
       <c r="A87" s="2">
         <v>83</v>
       </c>
-      <c r="B87" s="52"/>
-      <c r="C87" s="52"/>
+      <c r="B87" s="53"/>
+      <c r="C87" s="53"/>
       <c r="D87" s="2" t="s">
         <v>101</v>
       </c>
@@ -4422,8 +4428,8 @@
     </row>
     <row r="88" spans="1:7" ht="20.25" customHeight="1">
       <c r="A88" s="2"/>
-      <c r="B88" s="52"/>
-      <c r="C88" s="52"/>
+      <c r="B88" s="53"/>
+      <c r="C88" s="53"/>
       <c r="D88" s="2" t="s">
         <v>101</v>
       </c>
@@ -4436,8 +4442,8 @@
       <c r="A89" s="9">
         <v>84</v>
       </c>
-      <c r="B89" s="80"/>
-      <c r="C89" s="80"/>
+      <c r="B89" s="54"/>
+      <c r="C89" s="54"/>
       <c r="D89" s="9" t="s">
         <v>101</v>
       </c>
@@ -4938,7 +4944,7 @@
       <c r="B122" s="75">
         <v>46293</v>
       </c>
-      <c r="C122" s="63" t="s">
+      <c r="C122" s="64" t="s">
         <v>44</v>
       </c>
       <c r="D122" s="34" t="s">
@@ -4952,7 +4958,7 @@
     <row r="123" spans="1:6" ht="75">
       <c r="A123" s="34"/>
       <c r="B123" s="76"/>
-      <c r="C123" s="64"/>
+      <c r="C123" s="65"/>
       <c r="D123" s="34" t="s">
         <v>154</v>
       </c>
@@ -4964,7 +4970,7 @@
     <row r="124" spans="1:6">
       <c r="A124" s="34"/>
       <c r="B124" s="76"/>
-      <c r="C124" s="64"/>
+      <c r="C124" s="65"/>
       <c r="D124" s="34" t="s">
         <v>102</v>
       </c>
@@ -4976,7 +4982,7 @@
     <row r="125" spans="1:6">
       <c r="A125" s="34"/>
       <c r="B125" s="76"/>
-      <c r="C125" s="64"/>
+      <c r="C125" s="65"/>
       <c r="D125" s="34" t="s">
         <v>117</v>
       </c>
@@ -4988,7 +4994,7 @@
     <row r="126" spans="1:6">
       <c r="A126" s="34"/>
       <c r="B126" s="76"/>
-      <c r="C126" s="64"/>
+      <c r="C126" s="65"/>
       <c r="D126" s="34" t="s">
         <v>117</v>
       </c>
@@ -5000,7 +5006,7 @@
     <row r="127" spans="1:6">
       <c r="A127" s="34"/>
       <c r="B127" s="76"/>
-      <c r="C127" s="64"/>
+      <c r="C127" s="65"/>
       <c r="D127" s="34"/>
       <c r="E127" s="34"/>
       <c r="F127" s="34"/>
@@ -5008,7 +5014,7 @@
     <row r="128" spans="1:6">
       <c r="A128" s="34"/>
       <c r="B128" s="76"/>
-      <c r="C128" s="64"/>
+      <c r="C128" s="65"/>
       <c r="D128" s="34"/>
       <c r="E128" s="34"/>
       <c r="F128" s="34"/>
@@ -5016,7 +5022,7 @@
     <row r="129" spans="1:8" ht="165">
       <c r="A129" s="34"/>
       <c r="B129" s="76"/>
-      <c r="C129" s="64"/>
+      <c r="C129" s="65"/>
       <c r="D129" s="34"/>
       <c r="E129" s="35" t="s">
         <v>155</v>
@@ -5028,7 +5034,7 @@
     <row r="130" spans="1:8" ht="60">
       <c r="A130" s="34"/>
       <c r="B130" s="76"/>
-      <c r="C130" s="64"/>
+      <c r="C130" s="65"/>
       <c r="D130" s="34"/>
       <c r="E130" s="36" t="s">
         <v>157</v>
@@ -5038,7 +5044,7 @@
     <row r="131" spans="1:8">
       <c r="A131" s="34"/>
       <c r="B131" s="76"/>
-      <c r="C131" s="64"/>
+      <c r="C131" s="65"/>
       <c r="D131" s="34" t="s">
         <v>101</v>
       </c>
@@ -5050,7 +5056,7 @@
     <row r="132" spans="1:8">
       <c r="A132" s="34"/>
       <c r="B132" s="76"/>
-      <c r="C132" s="64"/>
+      <c r="C132" s="65"/>
       <c r="D132" s="34" t="s">
         <v>101</v>
       </c>
@@ -5062,7 +5068,7 @@
     <row r="133" spans="1:8">
       <c r="A133" s="34"/>
       <c r="B133" s="76"/>
-      <c r="C133" s="64"/>
+      <c r="C133" s="65"/>
       <c r="D133" s="34"/>
       <c r="E133" s="34" t="s">
         <v>160</v>
@@ -5072,7 +5078,7 @@
     <row r="134" spans="1:8" ht="45">
       <c r="A134" s="34"/>
       <c r="B134" s="76"/>
-      <c r="C134" s="64"/>
+      <c r="C134" s="65"/>
       <c r="D134" s="34" t="s">
         <v>129</v>
       </c>
@@ -5084,7 +5090,7 @@
     <row r="135" spans="1:8">
       <c r="A135" s="34"/>
       <c r="B135" s="76"/>
-      <c r="C135" s="64"/>
+      <c r="C135" s="65"/>
       <c r="D135" s="34"/>
       <c r="E135" s="34"/>
       <c r="F135" s="34"/>
@@ -5092,7 +5098,7 @@
     <row r="136" spans="1:8" ht="45">
       <c r="A136" s="34"/>
       <c r="B136" s="76"/>
-      <c r="C136" s="64"/>
+      <c r="C136" s="65"/>
       <c r="D136" s="34"/>
       <c r="E136" s="36" t="s">
         <v>162</v>
@@ -5104,7 +5110,7 @@
     <row r="137" spans="1:8" ht="45">
       <c r="A137" s="34"/>
       <c r="B137" s="77"/>
-      <c r="C137" s="65"/>
+      <c r="C137" s="66"/>
       <c r="D137" s="34"/>
       <c r="E137" s="35" t="s">
         <v>164</v>
@@ -5332,10 +5338,10 @@
     </row>
     <row r="159" spans="1:9">
       <c r="A159" s="22"/>
-      <c r="B159" s="57">
+      <c r="B159" s="58">
         <v>46302</v>
       </c>
-      <c r="C159" s="60" t="s">
+      <c r="C159" s="61" t="s">
         <v>215</v>
       </c>
       <c r="D159" s="22" t="s">
@@ -5348,8 +5354,8 @@
     </row>
     <row r="160" spans="1:9" ht="45">
       <c r="A160" s="22"/>
-      <c r="B160" s="58"/>
-      <c r="C160" s="61"/>
+      <c r="B160" s="59"/>
+      <c r="C160" s="62"/>
       <c r="D160" s="22" t="s">
         <v>111</v>
       </c>
@@ -5362,8 +5368,8 @@
     </row>
     <row r="161" spans="1:8" ht="45">
       <c r="A161" s="22"/>
-      <c r="B161" s="58"/>
-      <c r="C161" s="61"/>
+      <c r="B161" s="59"/>
+      <c r="C161" s="62"/>
       <c r="D161" s="22"/>
       <c r="E161" s="26" t="s">
         <v>203</v>
@@ -5374,8 +5380,8 @@
     </row>
     <row r="162" spans="1:8" ht="90">
       <c r="A162" s="22"/>
-      <c r="B162" s="58"/>
-      <c r="C162" s="61"/>
+      <c r="B162" s="59"/>
+      <c r="C162" s="62"/>
       <c r="D162" s="22"/>
       <c r="E162" s="26" t="s">
         <v>206</v>
@@ -5389,8 +5395,8 @@
     </row>
     <row r="163" spans="1:8" ht="60">
       <c r="A163" s="22"/>
-      <c r="B163" s="58"/>
-      <c r="C163" s="61"/>
+      <c r="B163" s="59"/>
+      <c r="C163" s="62"/>
       <c r="D163" s="22"/>
       <c r="E163" s="26" t="s">
         <v>210</v>
@@ -5404,8 +5410,8 @@
     </row>
     <row r="164" spans="1:8">
       <c r="A164" s="22"/>
-      <c r="B164" s="59"/>
-      <c r="C164" s="62"/>
+      <c r="B164" s="60"/>
+      <c r="C164" s="63"/>
       <c r="D164" s="22" t="s">
         <v>101</v>
       </c>
@@ -5738,28 +5744,49 @@
         <v>264</v>
       </c>
     </row>
+    <row r="232" spans="2:5">
+      <c r="D232" t="s">
+        <v>101</v>
+      </c>
+      <c r="E232" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="233" spans="2:5">
+      <c r="D233" t="s">
+        <v>111</v>
+      </c>
+      <c r="E233" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="234" spans="2:5">
+      <c r="B234" s="30">
+        <v>46322</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:F90" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="54">
-    <mergeCell ref="C78:C83"/>
-    <mergeCell ref="B84:B89"/>
-    <mergeCell ref="C84:C89"/>
-    <mergeCell ref="B67:B70"/>
-    <mergeCell ref="C67:C70"/>
-    <mergeCell ref="B71:B77"/>
-    <mergeCell ref="C71:C77"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B3:B7"/>
-    <mergeCell ref="C3:C7"/>
-    <mergeCell ref="D3:D7"/>
-    <mergeCell ref="B8:B16"/>
-    <mergeCell ref="C8:C16"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="B21:B25"/>
-    <mergeCell ref="C21:C25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="D71:D77"/>
+    <mergeCell ref="B39:B45"/>
+    <mergeCell ref="C39:C45"/>
+    <mergeCell ref="D39:D45"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="C46:C49"/>
+    <mergeCell ref="B52:B57"/>
+    <mergeCell ref="C52:C57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="C58:C61"/>
+    <mergeCell ref="B62:B66"/>
+    <mergeCell ref="C62:C66"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="D30:D33"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="C34:C38"/>
+    <mergeCell ref="D34:D38"/>
     <mergeCell ref="A50:A51"/>
     <mergeCell ref="B50:B51"/>
     <mergeCell ref="C50:C51"/>
@@ -5776,25 +5803,25 @@
     <mergeCell ref="C90:C94"/>
     <mergeCell ref="B90:B95"/>
     <mergeCell ref="B78:B83"/>
-    <mergeCell ref="D26:D29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="D30:D33"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="C34:C38"/>
-    <mergeCell ref="D34:D38"/>
-    <mergeCell ref="D71:D77"/>
-    <mergeCell ref="B39:B45"/>
-    <mergeCell ref="C39:C45"/>
-    <mergeCell ref="D39:D45"/>
-    <mergeCell ref="B46:B49"/>
-    <mergeCell ref="C46:C49"/>
-    <mergeCell ref="B52:B57"/>
-    <mergeCell ref="C52:C57"/>
-    <mergeCell ref="B58:B61"/>
-    <mergeCell ref="C58:C61"/>
-    <mergeCell ref="B62:B66"/>
-    <mergeCell ref="C62:C66"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="C21:C25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B3:B7"/>
+    <mergeCell ref="C3:C7"/>
+    <mergeCell ref="D3:D7"/>
+    <mergeCell ref="B8:B16"/>
+    <mergeCell ref="C8:C16"/>
+    <mergeCell ref="C78:C83"/>
+    <mergeCell ref="B84:B89"/>
+    <mergeCell ref="C84:C89"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="C67:C70"/>
+    <mergeCell ref="B71:B77"/>
+    <mergeCell ref="C71:C77"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>